<commit_message>
ajustando a janela dos input dos dados que não estava aparecendo
</commit_message>
<xml_diff>
--- a/laudo/templates/template_xlsx.xlsx
+++ b/laudo/templates/template_xlsx.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\documentos\automacao_extracao_pericia\laudo\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F5EC3C4-05A5-4826-B86C-7D34D27D3797}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9008543-AD19-4837-BC5D-56BE6BE1EEAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -314,7 +314,7 @@
     <numFmt numFmtId="169" formatCode="#,##0.00000000"/>
     <numFmt numFmtId="170" formatCode="&quot;R$ &quot;#,##0.00"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -417,8 +417,13 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <name val="Arial Narrow"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -435,6 +440,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFCCFFFF"/>
         <bgColor rgb="FFCCFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -632,16 +643,10 @@
     <xf numFmtId="165" fontId="14" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="165" fontId="14" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="130">
+  <cellXfs count="132">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="4" fontId="7" fillId="0" borderId="3" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="6" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="6" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="166" fontId="5" fillId="2" borderId="1" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -812,9 +817,6 @@
     <xf numFmtId="4" fontId="12" fillId="2" borderId="0" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="6" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="166" fontId="12" fillId="2" borderId="3" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -994,6 +996,21 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="25" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="6" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="6" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="7" fillId="0" borderId="3" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="15" fillId="4" borderId="3" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="4" fontId="15" fillId="0" borderId="3" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="41">
@@ -1449,68 +1466,68 @@
   </cols>
   <sheetData>
     <row r="9" spans="6:9">
-      <c r="F9" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="G9" s="5" t="s">
+      <c r="F9" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G9" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="H9" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="I9" s="7" t="s">
+      <c r="I9" s="5" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="10" spans="6:9">
-      <c r="F10" s="8">
+      <c r="F10" s="6">
         <v>44739</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="G10" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="H10" s="10">
+      <c r="H10" s="8">
         <v>1146.81</v>
       </c>
-      <c r="I10" s="11">
+      <c r="I10" s="9">
         <f>H10</f>
         <v>1146.81</v>
       </c>
     </row>
     <row r="11" spans="6:9">
-      <c r="F11" s="12">
+      <c r="F11" s="10">
         <v>44740</v>
       </c>
-      <c r="G11" s="13" t="s">
+      <c r="G11" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="H11" s="14">
+      <c r="H11" s="12">
         <v>2162.0300000000002</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="129">
         <f>H11+H12</f>
         <v>4093.05</v>
       </c>
     </row>
     <row r="12" spans="6:9">
-      <c r="F12" s="12">
+      <c r="F12" s="10">
         <v>45111</v>
       </c>
-      <c r="G12" s="13" t="s">
+      <c r="G12" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="H12" s="14">
+      <c r="H12" s="12">
         <v>1931.02</v>
       </c>
-      <c r="I12" s="1"/>
+      <c r="I12" s="129"/>
     </row>
     <row r="13" spans="6:9">
-      <c r="F13" s="15" t="s">
+      <c r="F13" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="G13" s="15"/>
-      <c r="H13" s="15"/>
-      <c r="I13" s="16">
+      <c r="G13" s="13"/>
+      <c r="H13" s="13"/>
+      <c r="I13" s="14">
         <f>SUM(I10:I12)</f>
         <v>5239.8600000000006</v>
       </c>
@@ -1533,1203 +1550,1224 @@
   <dimension ref="A1:AMK71"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="10.5703125" style="17" customWidth="1"/>
-    <col min="2" max="2" width="20.28515625" style="18" customWidth="1"/>
-    <col min="3" max="3" width="10.140625" style="19" customWidth="1"/>
-    <col min="4" max="4" width="10.42578125" style="20" customWidth="1"/>
-    <col min="5" max="5" width="9.5703125" style="19" customWidth="1"/>
-    <col min="6" max="6" width="1" style="21" customWidth="1"/>
-    <col min="7" max="7" width="9" style="22" customWidth="1"/>
-    <col min="8" max="8" width="12.85546875" style="22" customWidth="1"/>
-    <col min="9" max="9" width="9.7109375" style="23" customWidth="1"/>
-    <col min="10" max="10" width="8.28515625" style="23" customWidth="1"/>
-    <col min="11" max="11" width="10.7109375" style="24" customWidth="1"/>
-    <col min="12" max="12" width="10.7109375" style="23" customWidth="1"/>
-    <col min="13" max="13" width="10.7109375" style="25" customWidth="1"/>
-    <col min="14" max="14" width="10.7109375" style="22" customWidth="1"/>
-    <col min="15" max="15" width="66.42578125" style="26" customWidth="1"/>
-    <col min="16" max="16" width="10.7109375" style="20" customWidth="1"/>
-    <col min="17" max="18" width="10.7109375" style="19" customWidth="1"/>
-    <col min="19" max="20" width="10.7109375" style="19" hidden="1" customWidth="1"/>
-    <col min="21" max="22" width="10.7109375" style="19" customWidth="1"/>
-    <col min="23" max="23" width="10.7109375" style="20" customWidth="1"/>
-    <col min="24" max="24" width="6.5703125" style="27" customWidth="1"/>
-    <col min="25" max="1025" width="9.140625" style="28"/>
+    <col min="1" max="1" width="10.5703125" style="15" customWidth="1"/>
+    <col min="2" max="2" width="20.28515625" style="16" customWidth="1"/>
+    <col min="3" max="3" width="10.140625" style="17" customWidth="1"/>
+    <col min="4" max="4" width="10.42578125" style="18" customWidth="1"/>
+    <col min="5" max="5" width="9.5703125" style="17" customWidth="1"/>
+    <col min="6" max="6" width="1" style="19" customWidth="1"/>
+    <col min="7" max="7" width="9" style="20" customWidth="1"/>
+    <col min="8" max="8" width="12.85546875" style="20" customWidth="1"/>
+    <col min="9" max="9" width="9.7109375" style="21" customWidth="1"/>
+    <col min="10" max="10" width="8.28515625" style="21" customWidth="1"/>
+    <col min="11" max="11" width="10.7109375" style="22" customWidth="1"/>
+    <col min="12" max="12" width="10.7109375" style="21" customWidth="1"/>
+    <col min="13" max="13" width="10.7109375" style="23" customWidth="1"/>
+    <col min="14" max="14" width="10.7109375" style="20" customWidth="1"/>
+    <col min="15" max="15" width="66.42578125" style="24" customWidth="1"/>
+    <col min="16" max="16" width="10.7109375" style="18" customWidth="1"/>
+    <col min="17" max="18" width="10.7109375" style="17" customWidth="1"/>
+    <col min="19" max="20" width="10.7109375" style="17" hidden="1" customWidth="1"/>
+    <col min="21" max="22" width="10.7109375" style="17" customWidth="1"/>
+    <col min="23" max="23" width="10.7109375" style="18" customWidth="1"/>
+    <col min="24" max="24" width="6.5703125" style="25" customWidth="1"/>
+    <col min="25" max="1025" width="9.140625" style="26"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:31">
-      <c r="A1" s="29" t="str">
+      <c r="A1" s="27" t="str">
         <f>"Recálculo da operação nº "&amp;AA1&amp;" - Capitalização "&amp;AA2</f>
         <v>Recálculo da operação nº 409.906.274 - Capitalização Afastada</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="31"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="34"/>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
-      <c r="K1" s="32"/>
-      <c r="L1" s="31"/>
-      <c r="M1" s="35"/>
-      <c r="N1" s="34"/>
-      <c r="O1" s="36"/>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="31"/>
-      <c r="R1" s="31"/>
-      <c r="S1" s="31"/>
-      <c r="T1" s="31"/>
-      <c r="U1" s="31"/>
-      <c r="V1" s="31"/>
-      <c r="W1" s="32"/>
-      <c r="Y1" s="28">
+      <c r="B1" s="28"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="29"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="30"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="33"/>
+      <c r="N1" s="32"/>
+      <c r="O1" s="34"/>
+      <c r="P1" s="30"/>
+      <c r="Q1" s="29"/>
+      <c r="R1" s="29"/>
+      <c r="S1" s="29"/>
+      <c r="T1" s="29"/>
+      <c r="U1" s="29"/>
+      <c r="V1" s="29"/>
+      <c r="W1" s="30"/>
+      <c r="Y1" s="26">
         <f ca="1">_xlfn.SHEET()</f>
         <v>2</v>
       </c>
-      <c r="Z1" s="28" t="s">
+      <c r="Z1" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="AA1" s="37" t="s">
+      <c r="AA1" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="AB1" s="28" t="s">
+      <c r="AB1" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="AC1" s="28" t="s">
+      <c r="AC1" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="AD1" s="28" t="s">
+      <c r="AD1" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="AE1" s="28" t="s">
+      <c r="AE1" s="26" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:31">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="33"/>
-      <c r="H2" s="34"/>
-      <c r="I2" s="31"/>
-      <c r="J2" s="31"/>
-      <c r="K2" s="39" t="s">
+      <c r="G2" s="31"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="29"/>
+      <c r="J2" s="29"/>
+      <c r="K2" s="37" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="31"/>
-      <c r="M2" s="35"/>
-      <c r="N2" s="34"/>
-      <c r="O2" s="40"/>
-      <c r="P2" s="41"/>
-      <c r="Q2" s="42"/>
-      <c r="R2" s="42"/>
-      <c r="S2" s="42"/>
-      <c r="T2" s="42"/>
-      <c r="U2" s="42"/>
-      <c r="V2" s="31"/>
-      <c r="W2" s="32"/>
-      <c r="Z2" s="28" t="s">
+      <c r="L2" s="29"/>
+      <c r="M2" s="33"/>
+      <c r="N2" s="32"/>
+      <c r="O2" s="38"/>
+      <c r="P2" s="39"/>
+      <c r="Q2" s="40"/>
+      <c r="R2" s="40"/>
+      <c r="S2" s="40"/>
+      <c r="T2" s="40"/>
+      <c r="U2" s="40"/>
+      <c r="V2" s="29"/>
+      <c r="W2" s="30"/>
+      <c r="Z2" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="AA2" s="37" t="str">
+      <c r="AA2" s="35" t="str">
         <f>AD1</f>
         <v>Afastada</v>
       </c>
-      <c r="AB2" s="28" t="s">
+      <c r="AB2" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="AC2" s="28" t="s">
+      <c r="AC2" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="AD2" s="28" t="s">
+      <c r="AD2" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="AE2" s="28" t="s">
+      <c r="AE2" s="26" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:31">
-      <c r="A3" s="43" t="s">
+      <c r="A3" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B3" s="44">
+      <c r="B3" s="42">
         <f>SUMIF($B$13:$B$19,#REF!,$C$13:$C$19)</f>
         <v>0</v>
       </c>
-      <c r="C3" s="43" t="s">
+      <c r="C3" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="G3" s="33"/>
-      <c r="H3" s="34"/>
-      <c r="I3" s="31"/>
-      <c r="J3" s="31"/>
-      <c r="K3" s="45" t="str">
+      <c r="G3" s="31"/>
+      <c r="H3" s="32"/>
+      <c r="I3" s="29"/>
+      <c r="J3" s="29"/>
+      <c r="K3" s="43" t="str">
         <f>HLOOKUP(AA2,$AB$1:$AE$2,2,)</f>
         <v>Afastamento da capitalização de juros remuneratórios de normalidade</v>
       </c>
-      <c r="L3" s="31"/>
-      <c r="M3" s="35"/>
-      <c r="N3" s="34"/>
-      <c r="O3" s="46"/>
-      <c r="P3" s="47"/>
-      <c r="Q3" s="48"/>
-      <c r="R3" s="48"/>
-      <c r="S3" s="48"/>
-      <c r="T3" s="48"/>
-      <c r="U3" s="48"/>
-      <c r="V3" s="31"/>
-      <c r="W3" s="32"/>
-      <c r="Z3" s="37" t="s">
+      <c r="L3" s="29"/>
+      <c r="M3" s="33"/>
+      <c r="N3" s="32"/>
+      <c r="O3" s="44"/>
+      <c r="P3" s="45"/>
+      <c r="Q3" s="46"/>
+      <c r="R3" s="46"/>
+      <c r="S3" s="46"/>
+      <c r="T3" s="46"/>
+      <c r="U3" s="46"/>
+      <c r="V3" s="29"/>
+      <c r="W3" s="30"/>
+      <c r="Z3" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="AA3" s="28" t="str">
+      <c r="AA3" s="26" t="str">
         <f>IF(Z3="Execução","executado","cobrado")</f>
         <v>executado</v>
       </c>
-      <c r="AB3" s="28" t="str">
+      <c r="AB3" s="26" t="str">
         <f>IF(Z3="execução","execução","cobrança")</f>
         <v>execução</v>
       </c>
     </row>
     <row r="4" spans="1:31">
-      <c r="A4" s="43" t="s">
+      <c r="A4" s="41" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="44">
+      <c r="B4" s="42">
         <f>SUMIF($B$13:$B$19,#REF!,$C$13:$C$19)</f>
         <v>0</v>
       </c>
-      <c r="C4" s="44" t="s">
+      <c r="C4" s="42" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="49">
+      <c r="D4" s="47">
         <v>5.5E-2</v>
       </c>
-      <c r="E4" s="50" t="s">
+      <c r="E4" s="48" t="s">
         <v>25</v>
       </c>
-      <c r="G4" s="33"/>
-      <c r="H4" s="33"/>
-      <c r="I4" s="51"/>
-      <c r="J4" s="51"/>
-      <c r="K4" s="26" t="s">
+      <c r="G4" s="31"/>
+      <c r="H4" s="31"/>
+      <c r="I4" s="49"/>
+      <c r="J4" s="49"/>
+      <c r="K4" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="L4" s="51"/>
-      <c r="M4" s="52"/>
-      <c r="N4" s="33"/>
-      <c r="O4" s="46"/>
-      <c r="P4" s="47"/>
-      <c r="Q4" s="48"/>
-      <c r="R4" s="48"/>
-      <c r="S4" s="48"/>
-      <c r="T4" s="48"/>
-      <c r="U4" s="48"/>
-      <c r="V4" s="31"/>
-      <c r="W4" s="32"/>
+      <c r="L4" s="49"/>
+      <c r="M4" s="50"/>
+      <c r="N4" s="31"/>
+      <c r="O4" s="44"/>
+      <c r="P4" s="45"/>
+      <c r="Q4" s="46"/>
+      <c r="R4" s="46"/>
+      <c r="S4" s="46"/>
+      <c r="T4" s="46"/>
+      <c r="U4" s="46"/>
+      <c r="V4" s="29"/>
+      <c r="W4" s="30"/>
     </row>
     <row r="5" spans="1:31">
-      <c r="A5" s="28" t="s">
+      <c r="A5" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="B5" s="44" t="s">
+      <c r="B5" s="42" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="49">
+      <c r="D5" s="47">
         <f>(1+D4)^(1/12)-1</f>
         <v>4.471698917043021E-3</v>
       </c>
-      <c r="E5" s="50" t="s">
+      <c r="E5" s="48" t="s">
         <v>29</v>
       </c>
-      <c r="G5" s="33"/>
-      <c r="H5" s="33"/>
-      <c r="I5" s="51"/>
-      <c r="J5" s="51"/>
-      <c r="K5" s="43" t="s">
+      <c r="G5" s="31"/>
+      <c r="H5" s="31"/>
+      <c r="I5" s="49"/>
+      <c r="J5" s="49"/>
+      <c r="K5" s="41" t="s">
         <v>30</v>
       </c>
-      <c r="L5" s="51"/>
-      <c r="M5" s="52"/>
-      <c r="N5" s="33"/>
-      <c r="O5" s="36"/>
-      <c r="P5" s="32"/>
-      <c r="Q5" s="31"/>
-      <c r="R5" s="31"/>
-      <c r="S5" s="31"/>
-      <c r="T5" s="31"/>
-      <c r="U5" s="31"/>
-      <c r="V5" s="31"/>
-      <c r="W5" s="32"/>
+      <c r="L5" s="49"/>
+      <c r="M5" s="50"/>
+      <c r="N5" s="31"/>
+      <c r="O5" s="34"/>
+      <c r="P5" s="30"/>
+      <c r="Q5" s="29"/>
+      <c r="R5" s="29"/>
+      <c r="S5" s="29"/>
+      <c r="T5" s="29"/>
+      <c r="U5" s="29"/>
+      <c r="V5" s="29"/>
+      <c r="W5" s="30"/>
     </row>
     <row r="6" spans="1:31" ht="13.5" customHeight="1">
-      <c r="A6" s="43" t="s">
+      <c r="A6" s="41" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="44">
+      <c r="B6" s="42">
         <f>SUMIF($B$13:$B$19,#REF!,$C$13:$C$19)</f>
         <v>0</v>
       </c>
-      <c r="C6" s="43" t="s">
+      <c r="C6" s="41" t="s">
         <v>32</v>
       </c>
-      <c r="D6" s="44">
+      <c r="D6" s="42">
         <f>SUMIF($B$13:$B$19,#REF!,$C$13:$C$19)</f>
         <v>0</v>
       </c>
-      <c r="E6" s="50"/>
-      <c r="K6" s="45"/>
+      <c r="E6" s="48"/>
+      <c r="K6" s="43"/>
     </row>
     <row r="7" spans="1:31" ht="13.5" hidden="1" customHeight="1">
-      <c r="A7" s="43" t="s">
+      <c r="A7" s="41" t="s">
         <v>33</v>
       </c>
-      <c r="B7" s="44">
-        <v>0</v>
-      </c>
-      <c r="D7" s="49"/>
-      <c r="E7" s="50"/>
-      <c r="K7" s="45"/>
+      <c r="B7" s="42">
+        <v>0</v>
+      </c>
+      <c r="D7" s="47"/>
+      <c r="E7" s="48"/>
+      <c r="K7" s="43"/>
     </row>
     <row r="8" spans="1:31" ht="13.5" hidden="1" customHeight="1">
-      <c r="A8" s="43" t="s">
+      <c r="A8" s="41" t="s">
         <v>34</v>
       </c>
-      <c r="B8" s="44">
-        <v>0</v>
-      </c>
-      <c r="D8" s="49"/>
-      <c r="E8" s="50"/>
-      <c r="K8" s="45"/>
+      <c r="B8" s="42">
+        <v>0</v>
+      </c>
+      <c r="D8" s="47"/>
+      <c r="E8" s="48"/>
+      <c r="K8" s="43"/>
     </row>
     <row r="9" spans="1:31" ht="13.5" hidden="1" customHeight="1">
-      <c r="C9" s="28"/>
-      <c r="D9" s="28"/>
-      <c r="E9" s="28"/>
-    </row>
-    <row r="10" spans="1:31" s="63" customFormat="1" ht="5.25" customHeight="1">
-      <c r="A10" s="53"/>
-      <c r="B10" s="54"/>
-      <c r="C10" s="55"/>
-      <c r="D10" s="56"/>
-      <c r="E10" s="55"/>
-      <c r="F10" s="21"/>
-      <c r="G10" s="57"/>
-      <c r="H10" s="57"/>
-      <c r="I10" s="58"/>
-      <c r="J10" s="58"/>
-      <c r="K10" s="59"/>
-      <c r="L10" s="58"/>
-      <c r="M10" s="60"/>
-      <c r="N10" s="57"/>
-      <c r="O10" s="61"/>
-      <c r="P10" s="56"/>
-      <c r="Q10" s="55"/>
-      <c r="R10" s="55"/>
-      <c r="S10" s="55"/>
-      <c r="T10" s="55"/>
-      <c r="U10" s="55"/>
-      <c r="V10" s="55"/>
-      <c r="W10" s="56"/>
-      <c r="X10" s="62"/>
+      <c r="C9" s="26"/>
+      <c r="D9" s="26"/>
+      <c r="E9" s="26"/>
+    </row>
+    <row r="10" spans="1:31" s="61" customFormat="1" ht="5.25" customHeight="1">
+      <c r="A10" s="51"/>
+      <c r="B10" s="52"/>
+      <c r="C10" s="53"/>
+      <c r="D10" s="54"/>
+      <c r="E10" s="53"/>
+      <c r="F10" s="19"/>
+      <c r="G10" s="55"/>
+      <c r="H10" s="55"/>
+      <c r="I10" s="56"/>
+      <c r="J10" s="56"/>
+      <c r="K10" s="57"/>
+      <c r="L10" s="56"/>
+      <c r="M10" s="58"/>
+      <c r="N10" s="55"/>
+      <c r="O10" s="59"/>
+      <c r="P10" s="54"/>
+      <c r="Q10" s="53"/>
+      <c r="R10" s="53"/>
+      <c r="S10" s="53"/>
+      <c r="T10" s="53"/>
+      <c r="U10" s="53"/>
+      <c r="V10" s="53"/>
+      <c r="W10" s="54"/>
+      <c r="X10" s="60"/>
     </row>
     <row r="11" spans="1:31">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="127" t="s">
         <v>35</v>
       </c>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="64"/>
-      <c r="G11" s="2" t="s">
+      <c r="B11" s="127"/>
+      <c r="C11" s="127"/>
+      <c r="D11" s="127"/>
+      <c r="E11" s="127"/>
+      <c r="F11" s="62"/>
+      <c r="G11" s="128" t="s">
         <v>36</v>
       </c>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2"/>
-      <c r="K11" s="2"/>
-      <c r="L11" s="2"/>
-      <c r="M11" s="2"/>
-      <c r="N11" s="2"/>
-      <c r="O11" s="2"/>
-      <c r="P11" s="2"/>
-      <c r="Q11" s="2"/>
-      <c r="R11" s="2"/>
-      <c r="S11" s="2"/>
-      <c r="T11" s="2"/>
-      <c r="U11" s="2"/>
-      <c r="V11" s="2"/>
-      <c r="W11" s="2"/>
-    </row>
-    <row r="12" spans="1:31" s="72" customFormat="1" ht="27.75" customHeight="1">
-      <c r="A12" s="66" t="s">
-        <v>0</v>
-      </c>
-      <c r="B12" s="67" t="s">
+      <c r="H11" s="128"/>
+      <c r="I11" s="128"/>
+      <c r="J11" s="128"/>
+      <c r="K11" s="128"/>
+      <c r="L11" s="128"/>
+      <c r="M11" s="128"/>
+      <c r="N11" s="128"/>
+      <c r="O11" s="128"/>
+      <c r="P11" s="128"/>
+      <c r="Q11" s="128"/>
+      <c r="R11" s="128"/>
+      <c r="S11" s="128"/>
+      <c r="T11" s="128"/>
+      <c r="U11" s="128"/>
+      <c r="V11" s="128"/>
+      <c r="W11" s="128"/>
+    </row>
+    <row r="12" spans="1:31" s="69" customFormat="1" ht="27.75" customHeight="1">
+      <c r="A12" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B12" s="64" t="s">
         <v>1</v>
       </c>
-      <c r="C12" s="68" t="s">
+      <c r="C12" s="65" t="s">
         <v>2</v>
       </c>
-      <c r="D12" s="67" t="s">
+      <c r="D12" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="E12" s="68" t="s">
+      <c r="E12" s="65" t="s">
         <v>38</v>
       </c>
-      <c r="F12" s="69"/>
-      <c r="G12" s="67" t="s">
+      <c r="F12" s="66"/>
+      <c r="G12" s="64" t="s">
         <v>39</v>
       </c>
-      <c r="H12" s="67" t="s">
+      <c r="H12" s="64" t="s">
         <v>40</v>
       </c>
-      <c r="I12" s="68" t="s">
+      <c r="I12" s="65" t="s">
         <v>41</v>
       </c>
-      <c r="J12" s="68" t="s">
+      <c r="J12" s="65" t="s">
         <v>42</v>
       </c>
-      <c r="K12" s="67" t="s">
+      <c r="K12" s="64" t="s">
         <v>43</v>
       </c>
-      <c r="L12" s="68" t="s">
+      <c r="L12" s="65" t="s">
         <v>44</v>
       </c>
-      <c r="M12" s="70" t="s">
+      <c r="M12" s="67" t="s">
         <v>45</v>
       </c>
-      <c r="N12" s="67" t="s">
+      <c r="N12" s="64" t="s">
         <v>46</v>
       </c>
-      <c r="O12" s="67" t="s">
+      <c r="O12" s="64" t="s">
         <v>1</v>
       </c>
-      <c r="P12" s="67" t="s">
+      <c r="P12" s="64" t="s">
         <v>2</v>
       </c>
-      <c r="Q12" s="68" t="s">
+      <c r="Q12" s="65" t="s">
         <v>37</v>
       </c>
-      <c r="R12" s="68" t="s">
+      <c r="R12" s="65" t="s">
         <v>38</v>
       </c>
-      <c r="S12" s="68" t="s">
+      <c r="S12" s="65" t="s">
         <v>41</v>
       </c>
-      <c r="T12" s="68" t="s">
+      <c r="T12" s="65" t="s">
         <v>42</v>
       </c>
-      <c r="U12" s="68" t="s">
+      <c r="U12" s="65" t="s">
         <v>43</v>
       </c>
-      <c r="V12" s="68" t="s">
+      <c r="V12" s="65" t="s">
         <v>47</v>
       </c>
-      <c r="W12" s="67" t="s">
+      <c r="W12" s="64" t="s">
         <v>48</v>
       </c>
-      <c r="X12" s="71"/>
+      <c r="X12" s="68"/>
     </row>
     <row r="13" spans="1:31">
-      <c r="A13" s="73"/>
-      <c r="B13" s="74"/>
-      <c r="C13" s="75"/>
-      <c r="D13" s="75"/>
-      <c r="E13" s="75"/>
-      <c r="F13" s="77"/>
-      <c r="G13" s="78"/>
-      <c r="H13" s="78"/>
-      <c r="I13" s="79"/>
-      <c r="J13" s="79"/>
-      <c r="K13" s="80"/>
-      <c r="L13" s="80"/>
-      <c r="M13" s="81"/>
-      <c r="N13" s="90"/>
-      <c r="O13" s="82"/>
-      <c r="P13" s="88"/>
-      <c r="Q13" s="83"/>
-      <c r="R13" s="91"/>
-      <c r="S13" s="84"/>
-      <c r="T13" s="89"/>
-      <c r="U13" s="91"/>
-      <c r="V13" s="91"/>
-      <c r="W13" s="75"/>
-      <c r="X13" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="AC13" s="18" t="s">
+      <c r="A13" s="70"/>
+      <c r="B13" s="71"/>
+      <c r="C13" s="72"/>
+      <c r="D13" s="72"/>
+      <c r="E13" s="72"/>
+      <c r="F13" s="74"/>
+      <c r="G13" s="75"/>
+      <c r="H13" s="75"/>
+      <c r="I13" s="76"/>
+      <c r="J13" s="76"/>
+      <c r="K13" s="77"/>
+      <c r="L13" s="77"/>
+      <c r="M13" s="78"/>
+      <c r="N13" s="87"/>
+      <c r="O13" s="79"/>
+      <c r="P13" s="85"/>
+      <c r="Q13" s="80"/>
+      <c r="R13" s="88"/>
+      <c r="S13" s="81"/>
+      <c r="T13" s="86"/>
+      <c r="U13" s="88"/>
+      <c r="V13" s="88"/>
+      <c r="W13" s="130">
+        <f>V13</f>
+        <v>0</v>
+      </c>
+      <c r="X13" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="AC13" s="16" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:31">
-      <c r="A14" s="73"/>
-      <c r="B14" s="74"/>
-      <c r="C14" s="75"/>
-      <c r="D14" s="75"/>
-      <c r="E14" s="75"/>
-      <c r="F14" s="77"/>
-      <c r="G14" s="78"/>
-      <c r="H14" s="78"/>
-      <c r="I14" s="79"/>
-      <c r="J14" s="79"/>
-      <c r="K14" s="80"/>
-      <c r="L14" s="80"/>
-      <c r="M14" s="81"/>
-      <c r="N14" s="90"/>
-      <c r="O14" s="82"/>
-      <c r="P14" s="88"/>
-      <c r="Q14" s="83"/>
-      <c r="R14" s="91"/>
-      <c r="S14" s="84"/>
-      <c r="T14" s="89"/>
-      <c r="U14" s="91"/>
-      <c r="V14" s="91"/>
-      <c r="W14" s="75"/>
-      <c r="X14" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="AC14" s="28" t="s">
+      <c r="A14" s="70"/>
+      <c r="B14" s="71"/>
+      <c r="C14" s="72"/>
+      <c r="D14" s="72"/>
+      <c r="E14" s="72"/>
+      <c r="F14" s="74"/>
+      <c r="G14" s="75"/>
+      <c r="H14" s="75"/>
+      <c r="I14" s="76"/>
+      <c r="J14" s="76"/>
+      <c r="K14" s="77"/>
+      <c r="L14" s="77"/>
+      <c r="M14" s="78"/>
+      <c r="N14" s="87"/>
+      <c r="O14" s="79"/>
+      <c r="P14" s="85"/>
+      <c r="Q14" s="80"/>
+      <c r="R14" s="88"/>
+      <c r="S14" s="81"/>
+      <c r="T14" s="86"/>
+      <c r="U14" s="88"/>
+      <c r="V14" s="88"/>
+      <c r="W14" s="130">
+        <f>W13+V14</f>
+        <v>0</v>
+      </c>
+      <c r="X14" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="AC14" s="26" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="15" spans="1:31">
-      <c r="A15" s="73"/>
-      <c r="B15" s="74"/>
-      <c r="C15" s="75"/>
-      <c r="D15" s="75"/>
-      <c r="E15" s="75"/>
-      <c r="F15" s="77"/>
-      <c r="G15" s="78"/>
-      <c r="H15" s="78"/>
-      <c r="I15" s="79"/>
-      <c r="J15" s="79"/>
-      <c r="K15" s="80"/>
-      <c r="L15" s="80"/>
-      <c r="M15" s="81"/>
-      <c r="N15" s="90"/>
-      <c r="O15" s="82"/>
-      <c r="P15" s="88"/>
-      <c r="Q15" s="83"/>
-      <c r="R15" s="91"/>
-      <c r="S15" s="84"/>
-      <c r="T15" s="89"/>
-      <c r="U15" s="91"/>
-      <c r="V15" s="91"/>
-      <c r="W15" s="75"/>
-      <c r="X15" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="AC15" s="44" t="s">
+      <c r="A15" s="70"/>
+      <c r="B15" s="71"/>
+      <c r="C15" s="72"/>
+      <c r="D15" s="72"/>
+      <c r="E15" s="72"/>
+      <c r="F15" s="74"/>
+      <c r="G15" s="75"/>
+      <c r="H15" s="75"/>
+      <c r="I15" s="76"/>
+      <c r="J15" s="76"/>
+      <c r="K15" s="77"/>
+      <c r="L15" s="77"/>
+      <c r="M15" s="78"/>
+      <c r="N15" s="87"/>
+      <c r="O15" s="79"/>
+      <c r="P15" s="85"/>
+      <c r="Q15" s="80"/>
+      <c r="R15" s="88"/>
+      <c r="S15" s="81"/>
+      <c r="T15" s="86"/>
+      <c r="U15" s="88"/>
+      <c r="V15" s="88"/>
+      <c r="W15" s="130">
+        <f t="shared" ref="W15:W19" si="0">W14+V15</f>
+        <v>0</v>
+      </c>
+      <c r="X15" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="AC15" s="42" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="16" spans="1:31">
-      <c r="A16" s="73"/>
-      <c r="B16" s="74"/>
-      <c r="C16" s="75"/>
-      <c r="D16" s="75"/>
-      <c r="E16" s="75"/>
-      <c r="F16" s="77"/>
-      <c r="G16" s="78"/>
-      <c r="H16" s="78"/>
-      <c r="I16" s="79"/>
-      <c r="J16" s="79"/>
-      <c r="K16" s="80"/>
-      <c r="L16" s="80"/>
-      <c r="M16" s="81"/>
-      <c r="N16" s="90"/>
-      <c r="O16" s="82"/>
-      <c r="P16" s="88"/>
-      <c r="Q16" s="83"/>
-      <c r="R16" s="91"/>
-      <c r="S16" s="84"/>
-      <c r="T16" s="89"/>
-      <c r="U16" s="91"/>
-      <c r="V16" s="91"/>
-      <c r="W16" s="75"/>
-      <c r="X16" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Y16" s="18"/>
-      <c r="AC16" s="44" t="s">
+      <c r="A16" s="70"/>
+      <c r="B16" s="71"/>
+      <c r="C16" s="72"/>
+      <c r="D16" s="72"/>
+      <c r="E16" s="72"/>
+      <c r="F16" s="74"/>
+      <c r="G16" s="75"/>
+      <c r="H16" s="75"/>
+      <c r="I16" s="76"/>
+      <c r="J16" s="76"/>
+      <c r="K16" s="77"/>
+      <c r="L16" s="77"/>
+      <c r="M16" s="78"/>
+      <c r="N16" s="87"/>
+      <c r="O16" s="79"/>
+      <c r="P16" s="85"/>
+      <c r="Q16" s="80"/>
+      <c r="R16" s="88"/>
+      <c r="S16" s="81"/>
+      <c r="T16" s="86"/>
+      <c r="U16" s="88"/>
+      <c r="V16" s="88"/>
+      <c r="W16" s="131">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="X16" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="Y16" s="16"/>
+      <c r="AC16" s="42" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="17" spans="1:29">
-      <c r="A17" s="73"/>
-      <c r="B17" s="74"/>
-      <c r="C17" s="75"/>
-      <c r="D17" s="75"/>
-      <c r="E17" s="75"/>
-      <c r="F17" s="77"/>
-      <c r="G17" s="78"/>
-      <c r="H17" s="78"/>
-      <c r="I17" s="79"/>
-      <c r="J17" s="79"/>
-      <c r="K17" s="80"/>
-      <c r="L17" s="80"/>
-      <c r="M17" s="81"/>
-      <c r="N17" s="90"/>
-      <c r="O17" s="82"/>
-      <c r="P17" s="88"/>
-      <c r="Q17" s="83"/>
-      <c r="R17" s="91"/>
-      <c r="S17" s="84"/>
-      <c r="T17" s="89"/>
-      <c r="U17" s="91"/>
-      <c r="V17" s="91"/>
-      <c r="W17" s="75"/>
-      <c r="X17" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="AA17" s="92"/>
-      <c r="AC17" s="44" t="s">
+      <c r="A17" s="70"/>
+      <c r="B17" s="71"/>
+      <c r="C17" s="72"/>
+      <c r="D17" s="72"/>
+      <c r="E17" s="72"/>
+      <c r="F17" s="74"/>
+      <c r="G17" s="75"/>
+      <c r="H17" s="75"/>
+      <c r="I17" s="76"/>
+      <c r="J17" s="76"/>
+      <c r="K17" s="77"/>
+      <c r="L17" s="77"/>
+      <c r="M17" s="78"/>
+      <c r="N17" s="87"/>
+      <c r="O17" s="79"/>
+      <c r="P17" s="85"/>
+      <c r="Q17" s="80"/>
+      <c r="R17" s="88"/>
+      <c r="S17" s="81"/>
+      <c r="T17" s="86"/>
+      <c r="U17" s="88"/>
+      <c r="V17" s="88"/>
+      <c r="W17" s="131">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="X17" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="AA17" s="89"/>
+      <c r="AC17" s="42" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="18" spans="1:29">
-      <c r="A18" s="73"/>
-      <c r="B18" s="74"/>
-      <c r="C18" s="75"/>
-      <c r="D18" s="75"/>
-      <c r="E18" s="75"/>
-      <c r="F18" s="77"/>
-      <c r="G18" s="86"/>
-      <c r="H18" s="86"/>
-      <c r="I18" s="87"/>
-      <c r="J18" s="87"/>
-      <c r="K18" s="80"/>
-      <c r="L18" s="80"/>
-      <c r="M18" s="94"/>
-      <c r="N18" s="90"/>
-      <c r="O18" s="82"/>
-      <c r="P18" s="88"/>
-      <c r="Q18" s="83"/>
-      <c r="R18" s="91"/>
-      <c r="S18" s="84"/>
-      <c r="T18" s="89"/>
-      <c r="U18" s="91"/>
-      <c r="V18" s="91"/>
-      <c r="W18" s="75"/>
-      <c r="X18" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="AA18" s="85"/>
-      <c r="AC18" s="28" t="s">
+      <c r="A18" s="70"/>
+      <c r="B18" s="71"/>
+      <c r="C18" s="72"/>
+      <c r="D18" s="72"/>
+      <c r="E18" s="72"/>
+      <c r="F18" s="74"/>
+      <c r="G18" s="83"/>
+      <c r="H18" s="83"/>
+      <c r="I18" s="84"/>
+      <c r="J18" s="84"/>
+      <c r="K18" s="77"/>
+      <c r="L18" s="77"/>
+      <c r="M18" s="91"/>
+      <c r="N18" s="87"/>
+      <c r="O18" s="79"/>
+      <c r="P18" s="85"/>
+      <c r="Q18" s="80"/>
+      <c r="R18" s="88"/>
+      <c r="S18" s="81"/>
+      <c r="T18" s="86"/>
+      <c r="U18" s="88"/>
+      <c r="V18" s="88"/>
+      <c r="W18" s="131">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="X18" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="AA18" s="82"/>
+      <c r="AC18" s="26" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="19" spans="1:29">
-      <c r="A19" s="73"/>
-      <c r="B19" s="74"/>
-      <c r="C19" s="75"/>
-      <c r="D19" s="75"/>
-      <c r="E19" s="75"/>
-      <c r="F19" s="77"/>
-      <c r="G19" s="86"/>
-      <c r="H19" s="86"/>
-      <c r="I19" s="87"/>
-      <c r="J19" s="87"/>
-      <c r="K19" s="80"/>
-      <c r="L19" s="80"/>
-      <c r="M19" s="81"/>
-      <c r="N19" s="90"/>
-      <c r="O19" s="82"/>
-      <c r="P19" s="88"/>
-      <c r="Q19" s="83"/>
-      <c r="R19" s="91"/>
-      <c r="S19" s="84"/>
-      <c r="T19" s="89"/>
-      <c r="U19" s="91"/>
-      <c r="V19" s="91"/>
-      <c r="W19" s="75"/>
-      <c r="X19" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Z19" s="93"/>
-      <c r="AC19" s="18" t="s">
+      <c r="A19" s="70"/>
+      <c r="B19" s="71"/>
+      <c r="C19" s="72"/>
+      <c r="D19" s="72"/>
+      <c r="E19" s="72"/>
+      <c r="F19" s="74"/>
+      <c r="G19" s="83"/>
+      <c r="H19" s="83"/>
+      <c r="I19" s="84"/>
+      <c r="J19" s="84"/>
+      <c r="K19" s="77"/>
+      <c r="L19" s="77"/>
+      <c r="M19" s="78"/>
+      <c r="N19" s="87"/>
+      <c r="O19" s="79"/>
+      <c r="P19" s="85"/>
+      <c r="Q19" s="80"/>
+      <c r="R19" s="88"/>
+      <c r="S19" s="81"/>
+      <c r="T19" s="86"/>
+      <c r="U19" s="88"/>
+      <c r="V19" s="88"/>
+      <c r="W19" s="131">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="X19" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="Z19" s="90"/>
+      <c r="AC19" s="16" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:29">
-      <c r="A20" s="95"/>
-      <c r="B20" s="96" t="s">
+      <c r="A20" s="92"/>
+      <c r="B20" s="93" t="s">
         <v>56</v>
       </c>
-      <c r="C20" s="97"/>
-      <c r="D20" s="98"/>
-      <c r="E20" s="75">
+      <c r="C20" s="94"/>
+      <c r="D20" s="95"/>
+      <c r="E20" s="72">
         <f>E19-C20+D20</f>
         <v>0</v>
       </c>
-      <c r="F20" s="99"/>
-      <c r="G20" s="100"/>
-      <c r="H20" s="65"/>
-      <c r="I20" s="101"/>
-      <c r="J20" s="101"/>
-      <c r="K20" s="102"/>
-      <c r="L20" s="101"/>
-      <c r="M20" s="103"/>
-      <c r="N20" s="65"/>
-      <c r="O20" s="104" t="s">
+      <c r="F20" s="96"/>
+      <c r="G20" s="97"/>
+      <c r="H20" s="1"/>
+      <c r="I20" s="98"/>
+      <c r="J20" s="98"/>
+      <c r="K20" s="99"/>
+      <c r="L20" s="98"/>
+      <c r="M20" s="100"/>
+      <c r="N20" s="1"/>
+      <c r="O20" s="101" t="s">
         <v>57</v>
       </c>
-      <c r="P20" s="102"/>
-      <c r="Q20" s="105"/>
-      <c r="R20" s="91">
+      <c r="P20" s="99"/>
+      <c r="Q20" s="102"/>
+      <c r="R20" s="88">
         <f>R19-P20+Q20-C20+D20</f>
         <v>0</v>
       </c>
-      <c r="S20" s="106"/>
-      <c r="T20" s="107"/>
-      <c r="U20" s="107"/>
-      <c r="V20" s="42"/>
-      <c r="W20" s="42"/>
-      <c r="X20" s="85" t="e">
+      <c r="S20" s="103"/>
+      <c r="T20" s="104"/>
+      <c r="U20" s="104"/>
+      <c r="V20" s="40"/>
+      <c r="W20" s="40"/>
+      <c r="X20" s="82" t="e">
         <f>#REF!-#REF!</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="21" spans="1:29">
-      <c r="A21" s="95"/>
-      <c r="B21" s="30"/>
-      <c r="C21" s="31"/>
-      <c r="D21" s="32"/>
-      <c r="E21" s="31"/>
-      <c r="F21" s="31"/>
-      <c r="G21" s="33"/>
-      <c r="H21" s="33"/>
-      <c r="I21" s="51"/>
-      <c r="J21" s="51"/>
-      <c r="K21" s="108"/>
-      <c r="L21" s="51"/>
-      <c r="M21" s="52"/>
-      <c r="N21" s="33"/>
-      <c r="O21" s="36"/>
-      <c r="P21" s="31"/>
-      <c r="Q21" s="31"/>
-      <c r="R21" s="107"/>
-      <c r="S21" s="107"/>
-      <c r="T21" s="107"/>
-      <c r="U21" s="107"/>
-      <c r="V21" s="31"/>
-      <c r="W21" s="31"/>
-      <c r="X21" s="85" t="e">
+      <c r="A21" s="92"/>
+      <c r="B21" s="28"/>
+      <c r="C21" s="29"/>
+      <c r="D21" s="30"/>
+      <c r="E21" s="29"/>
+      <c r="F21" s="29"/>
+      <c r="G21" s="31"/>
+      <c r="H21" s="31"/>
+      <c r="I21" s="49"/>
+      <c r="J21" s="49"/>
+      <c r="K21" s="105"/>
+      <c r="L21" s="49"/>
+      <c r="M21" s="50"/>
+      <c r="N21" s="31"/>
+      <c r="O21" s="34"/>
+      <c r="P21" s="29"/>
+      <c r="Q21" s="29"/>
+      <c r="R21" s="104"/>
+      <c r="S21" s="104"/>
+      <c r="T21" s="104"/>
+      <c r="U21" s="104"/>
+      <c r="V21" s="29"/>
+      <c r="W21" s="29"/>
+      <c r="X21" s="82" t="e">
         <f>#REF!-#REF!</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="22" spans="1:29">
-      <c r="A22" s="95"/>
-      <c r="B22" s="109" t="s">
+      <c r="A22" s="92"/>
+      <c r="B22" s="106" t="s">
         <v>58</v>
       </c>
-      <c r="C22" s="110"/>
-      <c r="D22" s="111"/>
-      <c r="E22" s="110"/>
-      <c r="F22" s="112"/>
-      <c r="G22" s="65"/>
-      <c r="H22" s="65"/>
-      <c r="I22" s="101"/>
-      <c r="J22" s="101"/>
-      <c r="K22" s="102"/>
-      <c r="L22" s="101"/>
-      <c r="M22" s="103"/>
-      <c r="N22" s="65"/>
-      <c r="O22" s="113"/>
-      <c r="P22" s="114">
+      <c r="C22" s="107"/>
+      <c r="D22" s="108"/>
+      <c r="E22" s="107"/>
+      <c r="F22" s="109"/>
+      <c r="G22" s="1"/>
+      <c r="H22" s="1"/>
+      <c r="I22" s="98"/>
+      <c r="J22" s="98"/>
+      <c r="K22" s="99"/>
+      <c r="L22" s="98"/>
+      <c r="M22" s="100"/>
+      <c r="N22" s="1"/>
+      <c r="O22" s="110"/>
+      <c r="P22" s="111">
         <f>R20-E20</f>
         <v>0</v>
       </c>
-      <c r="Q22" s="31"/>
-      <c r="R22" s="31"/>
-      <c r="S22" s="31"/>
-      <c r="T22" s="31"/>
-      <c r="U22" s="31"/>
-      <c r="V22" s="31"/>
-      <c r="W22" s="32"/>
-      <c r="X22" s="85" t="e">
+      <c r="Q22" s="29"/>
+      <c r="R22" s="29"/>
+      <c r="S22" s="29"/>
+      <c r="T22" s="29"/>
+      <c r="U22" s="29"/>
+      <c r="V22" s="29"/>
+      <c r="W22" s="30"/>
+      <c r="X22" s="82" t="e">
         <f>#REF!-#REF!</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="23" spans="1:29">
-      <c r="A23" s="95"/>
-      <c r="B23" s="30"/>
-      <c r="C23" s="31"/>
-      <c r="D23" s="32"/>
-      <c r="E23" s="31"/>
-      <c r="G23" s="33"/>
-      <c r="H23" s="33"/>
-      <c r="I23" s="51"/>
-      <c r="J23" s="51"/>
-      <c r="K23" s="108"/>
-      <c r="L23" s="51"/>
-      <c r="M23" s="52"/>
-      <c r="N23" s="33"/>
-      <c r="O23" s="36"/>
-      <c r="P23" s="32"/>
-      <c r="Q23" s="31"/>
-      <c r="R23" s="31"/>
-      <c r="S23" s="31"/>
-      <c r="T23" s="31"/>
-      <c r="U23" s="31"/>
-      <c r="V23" s="31"/>
-      <c r="W23" s="32"/>
-      <c r="X23" s="85" t="e">
+      <c r="A23" s="92"/>
+      <c r="B23" s="28"/>
+      <c r="C23" s="29"/>
+      <c r="D23" s="30"/>
+      <c r="E23" s="29"/>
+      <c r="G23" s="31"/>
+      <c r="H23" s="31"/>
+      <c r="I23" s="49"/>
+      <c r="J23" s="49"/>
+      <c r="K23" s="105"/>
+      <c r="L23" s="49"/>
+      <c r="M23" s="50"/>
+      <c r="N23" s="31"/>
+      <c r="O23" s="34"/>
+      <c r="P23" s="30"/>
+      <c r="Q23" s="29"/>
+      <c r="R23" s="29"/>
+      <c r="S23" s="29"/>
+      <c r="T23" s="29"/>
+      <c r="U23" s="29"/>
+      <c r="V23" s="29"/>
+      <c r="W23" s="30"/>
+      <c r="X23" s="82" t="e">
         <f>#REF!-#REF!</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="24" spans="1:29">
-      <c r="A24" s="95"/>
-      <c r="B24" s="30"/>
-      <c r="C24" s="31"/>
-      <c r="D24" s="32"/>
-      <c r="E24" s="31"/>
-      <c r="G24" s="33"/>
-      <c r="H24" s="33"/>
-      <c r="I24" s="51"/>
-      <c r="J24" s="51"/>
-      <c r="K24" s="108"/>
-      <c r="L24" s="51"/>
-      <c r="M24" s="52"/>
-      <c r="N24" s="33"/>
-      <c r="O24" s="82" t="s">
+      <c r="A24" s="92"/>
+      <c r="B24" s="28"/>
+      <c r="C24" s="29"/>
+      <c r="D24" s="30"/>
+      <c r="E24" s="29"/>
+      <c r="G24" s="31"/>
+      <c r="H24" s="31"/>
+      <c r="I24" s="49"/>
+      <c r="J24" s="49"/>
+      <c r="K24" s="105"/>
+      <c r="L24" s="49"/>
+      <c r="M24" s="50"/>
+      <c r="N24" s="31"/>
+      <c r="O24" s="79" t="s">
         <v>59</v>
       </c>
-      <c r="P24" s="76">
+      <c r="P24" s="73">
         <f>R20</f>
         <v>0</v>
       </c>
-      <c r="Q24" s="31"/>
-      <c r="R24" s="31"/>
-      <c r="S24" s="31"/>
-      <c r="T24" s="31"/>
-      <c r="U24" s="31"/>
-      <c r="V24" s="31"/>
-      <c r="W24" s="32"/>
-      <c r="X24" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Y24" s="18"/>
+      <c r="Q24" s="29"/>
+      <c r="R24" s="29"/>
+      <c r="S24" s="29"/>
+      <c r="T24" s="29"/>
+      <c r="U24" s="29"/>
+      <c r="V24" s="29"/>
+      <c r="W24" s="30"/>
+      <c r="X24" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="Y24" s="16"/>
     </row>
     <row r="25" spans="1:29">
-      <c r="A25" s="95"/>
-      <c r="B25" s="30"/>
-      <c r="C25" s="31"/>
-      <c r="D25" s="32"/>
-      <c r="E25" s="31"/>
-      <c r="G25" s="33"/>
-      <c r="H25" s="33"/>
-      <c r="I25" s="51"/>
-      <c r="J25" s="51"/>
-      <c r="K25" s="108"/>
-      <c r="L25" s="51"/>
-      <c r="M25" s="52"/>
-      <c r="N25" s="33"/>
-      <c r="O25" s="82" t="str">
+      <c r="A25" s="92"/>
+      <c r="B25" s="28"/>
+      <c r="C25" s="29"/>
+      <c r="D25" s="30"/>
+      <c r="E25" s="29"/>
+      <c r="G25" s="31"/>
+      <c r="H25" s="31"/>
+      <c r="I25" s="49"/>
+      <c r="J25" s="49"/>
+      <c r="K25" s="105"/>
+      <c r="L25" s="49"/>
+      <c r="M25" s="50"/>
+      <c r="N25" s="31"/>
+      <c r="O25" s="79" t="str">
         <f>"Valor "&amp;AA3&amp;" (controverso):"</f>
         <v>Valor executado (controverso):</v>
       </c>
-      <c r="P25" s="76">
+      <c r="P25" s="73">
         <f>E20</f>
         <v>0</v>
       </c>
-      <c r="Q25" s="31"/>
-      <c r="R25" s="31"/>
-      <c r="S25" s="31"/>
-      <c r="T25" s="31"/>
-      <c r="U25" s="31"/>
-      <c r="V25" s="31"/>
-      <c r="W25" s="32"/>
-      <c r="X25" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Y25" s="18"/>
+      <c r="Q25" s="29"/>
+      <c r="R25" s="29"/>
+      <c r="S25" s="29"/>
+      <c r="T25" s="29"/>
+      <c r="U25" s="29"/>
+      <c r="V25" s="29"/>
+      <c r="W25" s="30"/>
+      <c r="X25" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="Y25" s="16"/>
     </row>
     <row r="26" spans="1:29">
-      <c r="A26" s="95"/>
-      <c r="B26" s="30"/>
-      <c r="C26" s="31"/>
-      <c r="D26" s="32"/>
-      <c r="E26" s="31"/>
-      <c r="G26" s="33"/>
-      <c r="H26" s="33"/>
-      <c r="I26" s="51"/>
-      <c r="J26" s="51"/>
-      <c r="K26" s="108"/>
-      <c r="L26" s="51"/>
-      <c r="M26" s="52"/>
-      <c r="N26" s="33"/>
-      <c r="O26" s="115" t="str">
+      <c r="A26" s="92"/>
+      <c r="B26" s="28"/>
+      <c r="C26" s="29"/>
+      <c r="D26" s="30"/>
+      <c r="E26" s="29"/>
+      <c r="G26" s="31"/>
+      <c r="H26" s="31"/>
+      <c r="I26" s="49"/>
+      <c r="J26" s="49"/>
+      <c r="K26" s="105"/>
+      <c r="L26" s="49"/>
+      <c r="M26" s="50"/>
+      <c r="N26" s="31"/>
+      <c r="O26" s="112" t="str">
         <f>"Excesso de "&amp;AB3&amp;":"</f>
         <v>Excesso de execução:</v>
       </c>
-      <c r="P26" s="116">
+      <c r="P26" s="113">
         <f>ABS(P24-P25)</f>
         <v>0</v>
       </c>
-      <c r="Q26" s="31"/>
-      <c r="R26" s="31"/>
-      <c r="S26" s="31"/>
-      <c r="T26" s="31"/>
-      <c r="U26" s="31"/>
-      <c r="V26" s="31"/>
-      <c r="W26" s="32"/>
-      <c r="X26" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Y26" s="18"/>
+      <c r="Q26" s="29"/>
+      <c r="R26" s="29"/>
+      <c r="S26" s="29"/>
+      <c r="T26" s="29"/>
+      <c r="U26" s="29"/>
+      <c r="V26" s="29"/>
+      <c r="W26" s="30"/>
+      <c r="X26" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="Y26" s="16"/>
     </row>
     <row r="27" spans="1:29">
-      <c r="A27" s="95"/>
-      <c r="B27" s="30"/>
-      <c r="C27" s="31"/>
-      <c r="D27" s="32"/>
-      <c r="E27" s="31"/>
-      <c r="G27" s="33"/>
-      <c r="H27" s="33"/>
-      <c r="I27" s="51"/>
-      <c r="J27" s="51"/>
-      <c r="K27" s="108"/>
-      <c r="L27" s="51"/>
-      <c r="M27" s="52"/>
-      <c r="N27" s="33"/>
-      <c r="O27" s="46" t="s">
+      <c r="A27" s="92"/>
+      <c r="B27" s="28"/>
+      <c r="C27" s="29"/>
+      <c r="D27" s="30"/>
+      <c r="E27" s="29"/>
+      <c r="G27" s="31"/>
+      <c r="H27" s="31"/>
+      <c r="I27" s="49"/>
+      <c r="J27" s="49"/>
+      <c r="K27" s="105"/>
+      <c r="L27" s="49"/>
+      <c r="M27" s="50"/>
+      <c r="N27" s="31"/>
+      <c r="O27" s="44" t="s">
         <v>60</v>
       </c>
-      <c r="P27" s="32"/>
-      <c r="Q27" s="31"/>
-      <c r="R27" s="31"/>
-      <c r="S27" s="31"/>
-      <c r="T27" s="31"/>
-      <c r="U27" s="31"/>
-      <c r="V27" s="31"/>
-      <c r="W27" s="32"/>
-      <c r="X27" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Y27" s="18"/>
+      <c r="P27" s="30"/>
+      <c r="Q27" s="29"/>
+      <c r="R27" s="29"/>
+      <c r="S27" s="29"/>
+      <c r="T27" s="29"/>
+      <c r="U27" s="29"/>
+      <c r="V27" s="29"/>
+      <c r="W27" s="30"/>
+      <c r="X27" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="Y27" s="16"/>
     </row>
     <row r="28" spans="1:29">
-      <c r="X28" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Y28" s="18"/>
+      <c r="X28" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="Y28" s="16"/>
     </row>
     <row r="29" spans="1:29">
-      <c r="B29" s="117" t="s">
+      <c r="B29" s="114" t="s">
         <v>61</v>
       </c>
-      <c r="C29" s="118"/>
-      <c r="D29" s="118"/>
-      <c r="E29" s="119">
+      <c r="C29" s="115"/>
+      <c r="D29" s="115"/>
+      <c r="E29" s="116">
         <f>E20</f>
         <v>0</v>
       </c>
-      <c r="O29" s="120" t="s">
+      <c r="O29" s="117" t="s">
         <v>62</v>
       </c>
-      <c r="P29" s="120"/>
-      <c r="Q29" s="120"/>
-      <c r="R29" s="118">
+      <c r="P29" s="117"/>
+      <c r="Q29" s="117"/>
+      <c r="R29" s="115">
         <f>R20</f>
         <v>0</v>
       </c>
-      <c r="X29" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Y29" s="18"/>
+      <c r="X29" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="Y29" s="16"/>
     </row>
     <row r="30" spans="1:29">
-      <c r="B30" s="117" t="s">
+      <c r="B30" s="114" t="s">
         <v>63</v>
       </c>
-      <c r="C30" s="118"/>
-      <c r="D30" s="118"/>
-      <c r="E30" s="121"/>
-      <c r="O30" s="117" t="s">
+      <c r="C30" s="115"/>
+      <c r="D30" s="115"/>
+      <c r="E30" s="118"/>
+      <c r="O30" s="114" t="s">
         <v>63</v>
       </c>
-      <c r="P30" s="120"/>
-      <c r="Q30" s="120"/>
-      <c r="R30" s="120">
+      <c r="P30" s="117"/>
+      <c r="Q30" s="117"/>
+      <c r="R30" s="117">
         <f>G30</f>
         <v>0</v>
       </c>
-      <c r="X30" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Y30" s="18"/>
+      <c r="X30" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="Y30" s="16"/>
     </row>
     <row r="31" spans="1:29">
-      <c r="B31" s="117" t="s">
+      <c r="B31" s="114" t="s">
         <v>65</v>
       </c>
-      <c r="C31" s="118"/>
-      <c r="D31" s="118"/>
-      <c r="E31" s="119">
+      <c r="C31" s="115"/>
+      <c r="D31" s="115"/>
+      <c r="E31" s="116">
         <f>E32-E29</f>
         <v>0</v>
       </c>
-      <c r="O31" s="117" t="s">
+      <c r="O31" s="114" t="s">
         <v>65</v>
       </c>
-      <c r="P31" s="120"/>
-      <c r="Q31" s="120"/>
-      <c r="R31" s="118">
+      <c r="P31" s="117"/>
+      <c r="Q31" s="117"/>
+      <c r="R31" s="115">
         <f>R32-R29</f>
         <v>0</v>
       </c>
-      <c r="X31" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Y31" s="18"/>
+      <c r="X31" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="Y31" s="16"/>
     </row>
     <row r="32" spans="1:29">
-      <c r="B32" s="117" t="s">
+      <c r="B32" s="114" t="s">
         <v>66</v>
       </c>
-      <c r="C32" s="118"/>
-      <c r="D32" s="118"/>
-      <c r="E32" s="119">
+      <c r="C32" s="115"/>
+      <c r="D32" s="115"/>
+      <c r="E32" s="116">
         <f>E29*E30</f>
         <v>0</v>
       </c>
-      <c r="O32" s="117" t="s">
+      <c r="O32" s="114" t="s">
         <v>67</v>
       </c>
-      <c r="P32" s="120"/>
-      <c r="Q32" s="120"/>
-      <c r="R32" s="118">
+      <c r="P32" s="117"/>
+      <c r="Q32" s="117"/>
+      <c r="R32" s="115">
         <f>R29*R30</f>
         <v>0</v>
       </c>
-      <c r="X32" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Y32" s="18"/>
+      <c r="X32" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="Y32" s="16"/>
     </row>
     <row r="33" spans="15:25">
-      <c r="O33" s="123"/>
-      <c r="P33" s="123"/>
-      <c r="Q33" s="123"/>
-      <c r="R33" s="124"/>
-      <c r="X33" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Y33" s="18"/>
+      <c r="O33" s="120"/>
+      <c r="P33" s="120"/>
+      <c r="Q33" s="120"/>
+      <c r="R33" s="121"/>
+      <c r="X33" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="Y33" s="16"/>
     </row>
     <row r="34" spans="15:25">
-      <c r="O34" s="126" t="s">
+      <c r="O34" s="123" t="s">
         <v>71</v>
       </c>
-      <c r="P34" s="126"/>
-      <c r="Q34" s="126"/>
-      <c r="R34" s="127">
+      <c r="P34" s="123"/>
+      <c r="Q34" s="123"/>
+      <c r="R34" s="124">
         <f>ABS(E32-R32)</f>
         <v>0</v>
       </c>
-      <c r="X34" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Y34" s="18"/>
+      <c r="X34" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="Y34" s="16"/>
     </row>
     <row r="35" spans="15:25">
-      <c r="O35" s="128" t="s">
+      <c r="O35" s="125" t="s">
         <v>60</v>
       </c>
-      <c r="P35" s="120"/>
-      <c r="Q35" s="120"/>
-      <c r="R35" s="118"/>
-      <c r="X35" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Y35" s="18"/>
+      <c r="P35" s="117"/>
+      <c r="Q35" s="117"/>
+      <c r="R35" s="115"/>
+      <c r="X35" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="Y35" s="16"/>
     </row>
     <row r="36" spans="15:25">
-      <c r="X36" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Y36" s="18"/>
+      <c r="X36" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="Y36" s="16"/>
     </row>
     <row r="37" spans="15:25">
-      <c r="O37" s="129" t="str">
+      <c r="O37" s="126" t="str">
         <f>"Excesso utilizado na operação nº xxxx - Anexo "</f>
         <v xml:space="preserve">Excesso utilizado na operação nº xxxx - Anexo </v>
       </c>
-      <c r="X37" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Y37" s="18"/>
+      <c r="X37" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="Y37" s="16"/>
     </row>
     <row r="38" spans="15:25">
-      <c r="X38" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Y38" s="18"/>
+      <c r="X38" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="Y38" s="16"/>
     </row>
     <row r="39" spans="15:25">
-      <c r="X39" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Y39" s="18"/>
+      <c r="X39" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="Y39" s="16"/>
     </row>
     <row r="40" spans="15:25">
-      <c r="X40" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Y40" s="18"/>
+      <c r="X40" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="Y40" s="16"/>
     </row>
     <row r="41" spans="15:25">
-      <c r="X41" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Y41" s="18"/>
+      <c r="X41" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="Y41" s="16"/>
     </row>
     <row r="42" spans="15:25">
-      <c r="X42" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Y42" s="18"/>
+      <c r="X42" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="Y42" s="16"/>
     </row>
     <row r="43" spans="15:25">
-      <c r="X43" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Y43" s="18"/>
+      <c r="X43" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="Y43" s="16"/>
     </row>
     <row r="44" spans="15:25">
-      <c r="X44" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Y44" s="18"/>
+      <c r="X44" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="Y44" s="16"/>
     </row>
     <row r="45" spans="15:25">
-      <c r="X45" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Y45" s="18"/>
+      <c r="X45" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="Y45" s="16"/>
     </row>
     <row r="46" spans="15:25">
-      <c r="X46" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Y46" s="18"/>
+      <c r="X46" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="Y46" s="16"/>
     </row>
     <row r="47" spans="15:25">
-      <c r="X47" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Y47" s="18"/>
+      <c r="X47" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="Y47" s="16"/>
     </row>
     <row r="48" spans="15:25">
-      <c r="X48" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Y48" s="18"/>
+      <c r="X48" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="Y48" s="16"/>
     </row>
     <row r="49" spans="24:25">
-      <c r="X49" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Y49" s="18"/>
+      <c r="X49" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="Y49" s="16"/>
     </row>
     <row r="50" spans="24:25">
-      <c r="X50" s="85" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Y50" s="18"/>
+      <c r="X50" s="82" t="e">
+        <f>#REF!-#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="Y50" s="16"/>
     </row>
     <row r="51" spans="24:25">
-      <c r="X51" s="85">
-        <f>V13-Q13</f>
-        <v>0</v>
-      </c>
-      <c r="Y51" s="18"/>
+      <c r="X51" s="82">
+        <f t="shared" ref="X51:X57" si="1">V13-Q13</f>
+        <v>0</v>
+      </c>
+      <c r="Y51" s="16"/>
     </row>
     <row r="52" spans="24:25">
-      <c r="X52" s="85">
-        <f>V14-Q14</f>
-        <v>0</v>
-      </c>
-      <c r="Y52" s="18"/>
+      <c r="X52" s="82">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y52" s="16"/>
     </row>
     <row r="53" spans="24:25">
-      <c r="X53" s="85">
-        <f>V15-Q15</f>
-        <v>0</v>
-      </c>
-      <c r="Y53" s="18"/>
+      <c r="X53" s="82">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y53" s="16"/>
     </row>
     <row r="54" spans="24:25">
-      <c r="X54" s="85">
-        <f>V16-Q16</f>
-        <v>0</v>
-      </c>
-      <c r="Y54" s="18"/>
+      <c r="X54" s="82">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y54" s="16"/>
     </row>
     <row r="55" spans="24:25">
-      <c r="X55" s="85">
-        <f>V17-Q17</f>
-        <v>0</v>
-      </c>
-      <c r="Y55" s="18"/>
+      <c r="X55" s="82">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y55" s="16"/>
     </row>
     <row r="56" spans="24:25">
-      <c r="X56" s="85">
-        <f>V18-Q18</f>
-        <v>0</v>
-      </c>
-      <c r="Y56" s="18"/>
+      <c r="X56" s="82">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y56" s="16"/>
     </row>
     <row r="57" spans="24:25">
-      <c r="X57" s="85">
-        <f>V19-Q19</f>
-        <v>0</v>
-      </c>
-      <c r="Y57" s="18"/>
+      <c r="X57" s="82">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y57" s="16"/>
     </row>
     <row r="58" spans="24:25">
-      <c r="X58" s="27" t="e">
+      <c r="X58" s="25" t="e">
         <f>SUM(X13:X57)</f>
         <v>#REF!</v>
       </c>
@@ -2737,28 +2775,28 @@
     <row r="60" spans="24:25" ht="13.5" hidden="1" customHeight="1"/>
     <row r="61" spans="24:25" ht="13.5" hidden="1" customHeight="1"/>
     <row r="68" spans="25:26">
-      <c r="Y68" s="122" t="s">
+      <c r="Y68" s="119" t="s">
         <v>64</v>
       </c>
-      <c r="Z68" s="122"/>
+      <c r="Z68" s="119"/>
     </row>
     <row r="69" spans="25:26">
-      <c r="Y69" s="122"/>
-      <c r="Z69" s="122"/>
+      <c r="Y69" s="119"/>
+      <c r="Z69" s="119"/>
     </row>
     <row r="70" spans="25:26">
-      <c r="Y70" s="122" t="s">
+      <c r="Y70" s="119" t="s">
         <v>68</v>
       </c>
-      <c r="Z70" s="122" t="s">
+      <c r="Z70" s="119" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="71" spans="25:26">
-      <c r="Y71" s="122" t="s">
+      <c r="Y71" s="119" t="s">
         <v>70</v>
       </c>
-      <c r="Z71" s="125" t="str">
+      <c r="Z71" s="122" t="str">
         <f>A1</f>
         <v>Recálculo da operação nº 409.906.274 - Capitalização Afastada</v>
       </c>

</xml_diff>

<commit_message>
ajuste de cabeçalho do excel
</commit_message>
<xml_diff>
--- a/laudo/templates/template_xlsx.xlsx
+++ b/laudo/templates/template_xlsx.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\documentos\automacao_extracao_pericia\laudo\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9008543-AD19-4837-BC5D-56BE6BE1EEAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21A7375E-6BB9-48C7-A88B-76DE2E86B1A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan" sheetId="1" r:id="rId1"/>
@@ -997,6 +997,12 @@
     <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="25" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="4" fontId="15" fillId="4" borderId="3" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="4" fontId="15" fillId="0" borderId="3" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="6" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1005,12 +1011,6 @@
     </xf>
     <xf numFmtId="4" fontId="7" fillId="0" borderId="3" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="15" fillId="4" borderId="3" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="4" fontId="15" fillId="0" borderId="3" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="41">
@@ -1504,7 +1504,7 @@
       <c r="H11" s="12">
         <v>2162.0300000000002</v>
       </c>
-      <c r="I11" s="129">
+      <c r="I11" s="131">
         <f>H11+H12</f>
         <v>4093.05</v>
       </c>
@@ -1519,7 +1519,7 @@
       <c r="H12" s="12">
         <v>1931.02</v>
       </c>
-      <c r="I12" s="129"/>
+      <c r="I12" s="131"/>
     </row>
     <row r="13" spans="6:9">
       <c r="F13" s="13" t="s">
@@ -1798,7 +1798,7 @@
       <c r="E6" s="48"/>
       <c r="K6" s="43"/>
     </row>
-    <row r="7" spans="1:31" ht="13.5" hidden="1" customHeight="1">
+    <row r="7" spans="1:31" ht="13.5" customHeight="1">
       <c r="A7" s="41" t="s">
         <v>33</v>
       </c>
@@ -1809,7 +1809,7 @@
       <c r="E7" s="48"/>
       <c r="K7" s="43"/>
     </row>
-    <row r="8" spans="1:31" ht="13.5" hidden="1" customHeight="1">
+    <row r="8" spans="1:31" ht="13.5" customHeight="1">
       <c r="A8" s="41" t="s">
         <v>34</v>
       </c>
@@ -1820,7 +1820,7 @@
       <c r="E8" s="48"/>
       <c r="K8" s="43"/>
     </row>
-    <row r="9" spans="1:31" ht="13.5" hidden="1" customHeight="1">
+    <row r="9" spans="1:31" ht="13.5" customHeight="1">
       <c r="C9" s="26"/>
       <c r="D9" s="26"/>
       <c r="E9" s="26"/>
@@ -1852,33 +1852,33 @@
       <c r="X10" s="60"/>
     </row>
     <row r="11" spans="1:31">
-      <c r="A11" s="127" t="s">
+      <c r="A11" s="129" t="s">
         <v>35</v>
       </c>
-      <c r="B11" s="127"/>
-      <c r="C11" s="127"/>
-      <c r="D11" s="127"/>
-      <c r="E11" s="127"/>
+      <c r="B11" s="129"/>
+      <c r="C11" s="129"/>
+      <c r="D11" s="129"/>
+      <c r="E11" s="129"/>
       <c r="F11" s="62"/>
-      <c r="G11" s="128" t="s">
+      <c r="G11" s="130" t="s">
         <v>36</v>
       </c>
-      <c r="H11" s="128"/>
-      <c r="I11" s="128"/>
-      <c r="J11" s="128"/>
-      <c r="K11" s="128"/>
-      <c r="L11" s="128"/>
-      <c r="M11" s="128"/>
-      <c r="N11" s="128"/>
-      <c r="O11" s="128"/>
-      <c r="P11" s="128"/>
-      <c r="Q11" s="128"/>
-      <c r="R11" s="128"/>
-      <c r="S11" s="128"/>
-      <c r="T11" s="128"/>
-      <c r="U11" s="128"/>
-      <c r="V11" s="128"/>
-      <c r="W11" s="128"/>
+      <c r="H11" s="130"/>
+      <c r="I11" s="130"/>
+      <c r="J11" s="130"/>
+      <c r="K11" s="130"/>
+      <c r="L11" s="130"/>
+      <c r="M11" s="130"/>
+      <c r="N11" s="130"/>
+      <c r="O11" s="130"/>
+      <c r="P11" s="130"/>
+      <c r="Q11" s="130"/>
+      <c r="R11" s="130"/>
+      <c r="S11" s="130"/>
+      <c r="T11" s="130"/>
+      <c r="U11" s="130"/>
+      <c r="V11" s="130"/>
+      <c r="W11" s="130"/>
     </row>
     <row r="12" spans="1:31" s="69" customFormat="1" ht="27.75" customHeight="1">
       <c r="A12" s="63" t="s">
@@ -1973,7 +1973,7 @@
       <c r="T13" s="86"/>
       <c r="U13" s="88"/>
       <c r="V13" s="88"/>
-      <c r="W13" s="130">
+      <c r="W13" s="127">
         <f>V13</f>
         <v>0</v>
       </c>
@@ -2008,7 +2008,7 @@
       <c r="T14" s="86"/>
       <c r="U14" s="88"/>
       <c r="V14" s="88"/>
-      <c r="W14" s="130">
+      <c r="W14" s="127">
         <f>W13+V14</f>
         <v>0</v>
       </c>
@@ -2043,7 +2043,7 @@
       <c r="T15" s="86"/>
       <c r="U15" s="88"/>
       <c r="V15" s="88"/>
-      <c r="W15" s="130">
+      <c r="W15" s="127">
         <f t="shared" ref="W15:W19" si="0">W14+V15</f>
         <v>0</v>
       </c>
@@ -2078,7 +2078,7 @@
       <c r="T16" s="86"/>
       <c r="U16" s="88"/>
       <c r="V16" s="88"/>
-      <c r="W16" s="131">
+      <c r="W16" s="128">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2114,7 +2114,7 @@
       <c r="T17" s="86"/>
       <c r="U17" s="88"/>
       <c r="V17" s="88"/>
-      <c r="W17" s="131">
+      <c r="W17" s="128">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2150,7 +2150,7 @@
       <c r="T18" s="86"/>
       <c r="U18" s="88"/>
       <c r="V18" s="88"/>
-      <c r="W18" s="131">
+      <c r="W18" s="128">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2186,7 +2186,7 @@
       <c r="T19" s="86"/>
       <c r="U19" s="88"/>
       <c r="V19" s="88"/>
-      <c r="W19" s="131">
+      <c r="W19" s="128">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
ajustar a estrutura do laudo
</commit_message>
<xml_diff>
--- a/laudo/templates/template_xlsx.xlsx
+++ b/laudo/templates/template_xlsx.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\documentos\automacao_extracao_pericia\laudo\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21A7375E-6BB9-48C7-A88B-76DE2E86B1A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E97C183E-C988-4C1B-9E03-1F94DBEAA5A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -314,7 +314,7 @@
     <numFmt numFmtId="169" formatCode="#,##0.00000000"/>
     <numFmt numFmtId="170" formatCode="&quot;R$ &quot;#,##0.00"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -422,8 +422,14 @@
       <name val="Arial Narrow"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <name val="Arial Narrow"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -446,6 +452,18 @@
       <patternFill patternType="solid">
         <fgColor theme="0"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCCFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFFCC"/>
       </patternFill>
     </fill>
   </fills>
@@ -643,7 +661,7 @@
     <xf numFmtId="165" fontId="14" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="165" fontId="14" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="132">
+  <cellXfs count="137">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="6" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -887,9 +905,6 @@
     <xf numFmtId="4" fontId="8" fillId="3" borderId="3" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="4" fontId="8" fillId="0" borderId="3" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
@@ -1011,6 +1026,24 @@
     </xf>
     <xf numFmtId="4" fontId="7" fillId="0" borderId="3" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="8" fillId="0" borderId="3" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="3" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="16" fillId="5" borderId="3" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="16" fillId="4" borderId="3" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="16" fillId="4" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="3" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="41">
@@ -1504,7 +1537,7 @@
       <c r="H11" s="12">
         <v>2162.0300000000002</v>
       </c>
-      <c r="I11" s="131">
+      <c r="I11" s="130">
         <f>H11+H12</f>
         <v>4093.05</v>
       </c>
@@ -1519,7 +1552,7 @@
       <c r="H12" s="12">
         <v>1931.02</v>
       </c>
-      <c r="I12" s="131"/>
+      <c r="I12" s="130"/>
     </row>
     <row r="13" spans="6:9">
       <c r="F13" s="13" t="s">
@@ -1571,7 +1604,8 @@
     <col min="21" max="22" width="10.7109375" style="17" customWidth="1"/>
     <col min="23" max="23" width="10.7109375" style="18" customWidth="1"/>
     <col min="24" max="24" width="6.5703125" style="25" customWidth="1"/>
-    <col min="25" max="1025" width="9.140625" style="26"/>
+    <col min="25" max="25" width="10.5703125" style="26" bestFit="1" customWidth="1"/>
+    <col min="26" max="1025" width="9.140625" style="26"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:31">
@@ -1791,7 +1825,7 @@
       <c r="C6" s="41" t="s">
         <v>32</v>
       </c>
-      <c r="D6" s="42">
+      <c r="D6" s="17">
         <f>SUMIF($B$13:$B$19,#REF!,$C$13:$C$19)</f>
         <v>0</v>
       </c>
@@ -1852,33 +1886,33 @@
       <c r="X10" s="60"/>
     </row>
     <row r="11" spans="1:31">
-      <c r="A11" s="129" t="s">
+      <c r="A11" s="128" t="s">
         <v>35</v>
       </c>
-      <c r="B11" s="129"/>
-      <c r="C11" s="129"/>
-      <c r="D11" s="129"/>
-      <c r="E11" s="129"/>
+      <c r="B11" s="128"/>
+      <c r="C11" s="128"/>
+      <c r="D11" s="128"/>
+      <c r="E11" s="128"/>
       <c r="F11" s="62"/>
-      <c r="G11" s="130" t="s">
+      <c r="G11" s="129" t="s">
         <v>36</v>
       </c>
-      <c r="H11" s="130"/>
-      <c r="I11" s="130"/>
-      <c r="J11" s="130"/>
-      <c r="K11" s="130"/>
-      <c r="L11" s="130"/>
-      <c r="M11" s="130"/>
-      <c r="N11" s="130"/>
-      <c r="O11" s="130"/>
-      <c r="P11" s="130"/>
-      <c r="Q11" s="130"/>
-      <c r="R11" s="130"/>
-      <c r="S11" s="130"/>
-      <c r="T11" s="130"/>
-      <c r="U11" s="130"/>
-      <c r="V11" s="130"/>
-      <c r="W11" s="130"/>
+      <c r="H11" s="129"/>
+      <c r="I11" s="129"/>
+      <c r="J11" s="129"/>
+      <c r="K11" s="129"/>
+      <c r="L11" s="129"/>
+      <c r="M11" s="129"/>
+      <c r="N11" s="129"/>
+      <c r="O11" s="129"/>
+      <c r="P11" s="129"/>
+      <c r="Q11" s="129"/>
+      <c r="R11" s="129"/>
+      <c r="S11" s="129"/>
+      <c r="T11" s="129"/>
+      <c r="U11" s="129"/>
+      <c r="V11" s="129"/>
+      <c r="W11" s="129"/>
     </row>
     <row r="12" spans="1:31" s="69" customFormat="1" ht="27.75" customHeight="1">
       <c r="A12" s="63" t="s">
@@ -1918,7 +1952,7 @@
       <c r="M12" s="67" t="s">
         <v>45</v>
       </c>
-      <c r="N12" s="64" t="s">
+      <c r="N12" s="136" t="s">
         <v>46</v>
       </c>
       <c r="O12" s="64" t="s">
@@ -1957,29 +1991,50 @@
       <c r="D13" s="72"/>
       <c r="E13" s="72"/>
       <c r="F13" s="74"/>
-      <c r="G13" s="75"/>
-      <c r="H13" s="75"/>
-      <c r="I13" s="76"/>
-      <c r="J13" s="76"/>
-      <c r="K13" s="77"/>
-      <c r="L13" s="77"/>
-      <c r="M13" s="78"/>
-      <c r="N13" s="87"/>
+      <c r="G13" s="132">
+        <f t="shared" ref="G13" si="0">_xlfn.DAYS(A14,A13)</f>
+        <v>0</v>
+      </c>
+      <c r="H13" s="132">
+        <f>G13</f>
+        <v>0</v>
+      </c>
+      <c r="I13" s="133">
+        <f t="shared" ref="I13" si="1">IF(E13&lt;0,G13*E13,0)</f>
+        <v>0</v>
+      </c>
+      <c r="J13" s="133">
+        <f>I13</f>
+        <v>0</v>
+      </c>
+      <c r="K13" s="134" t="e">
+        <f>ABS(J12/H12)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="L13" s="134">
+        <f>C13</f>
+        <v>0</v>
+      </c>
+      <c r="M13" s="135" t="e">
+        <f>(1+L13/K13)^(30/H12)-1</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="N13" s="131"/>
       <c r="O13" s="79"/>
       <c r="P13" s="85"/>
       <c r="Q13" s="80"/>
-      <c r="R13" s="88"/>
+      <c r="R13" s="87"/>
       <c r="S13" s="81"/>
       <c r="T13" s="86"/>
-      <c r="U13" s="88"/>
-      <c r="V13" s="88"/>
-      <c r="W13" s="127">
+      <c r="U13" s="87"/>
+      <c r="V13" s="87"/>
+      <c r="W13" s="126">
         <f>V13</f>
         <v>0</v>
       </c>
-      <c r="X13" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
+      <c r="X13" s="82">
+        <f>V13-Q13</f>
+        <v>0</v>
       </c>
       <c r="AC13" s="16" t="s">
         <v>49</v>
@@ -1999,22 +2054,26 @@
       <c r="K14" s="77"/>
       <c r="L14" s="77"/>
       <c r="M14" s="78"/>
-      <c r="N14" s="87"/>
+      <c r="N14" s="131"/>
       <c r="O14" s="79"/>
       <c r="P14" s="85"/>
       <c r="Q14" s="80"/>
-      <c r="R14" s="88"/>
+      <c r="R14" s="87"/>
       <c r="S14" s="81"/>
       <c r="T14" s="86"/>
-      <c r="U14" s="88"/>
-      <c r="V14" s="88"/>
-      <c r="W14" s="127">
+      <c r="U14" s="87"/>
+      <c r="V14" s="87"/>
+      <c r="W14" s="126">
         <f>W13+V14</f>
         <v>0</v>
       </c>
-      <c r="X14" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
+      <c r="X14" s="82">
+        <f t="shared" ref="X14:X19" si="2">V14-Q14</f>
+        <v>0</v>
+      </c>
+      <c r="Y14" s="26" t="b">
+        <f>ROUND(V14,2)=ROUND(L14,2)</f>
+        <v>1</v>
       </c>
       <c r="AC14" s="26" t="s">
         <v>50</v>
@@ -2034,22 +2093,26 @@
       <c r="K15" s="77"/>
       <c r="L15" s="77"/>
       <c r="M15" s="78"/>
-      <c r="N15" s="87"/>
+      <c r="N15" s="131"/>
       <c r="O15" s="79"/>
       <c r="P15" s="85"/>
       <c r="Q15" s="80"/>
-      <c r="R15" s="88"/>
+      <c r="R15" s="87"/>
       <c r="S15" s="81"/>
       <c r="T15" s="86"/>
-      <c r="U15" s="88"/>
-      <c r="V15" s="88"/>
-      <c r="W15" s="127">
-        <f t="shared" ref="W15:W19" si="0">W14+V15</f>
-        <v>0</v>
-      </c>
-      <c r="X15" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
+      <c r="U15" s="87"/>
+      <c r="V15" s="87"/>
+      <c r="W15" s="126">
+        <f t="shared" ref="W15:W19" si="3">W14+V15</f>
+        <v>0</v>
+      </c>
+      <c r="X15" s="82">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Y15" s="26" t="b">
+        <f t="shared" ref="Y15:Y19" si="4">ROUND(V15,2)=ROUND(L15,2)</f>
+        <v>1</v>
       </c>
       <c r="AC15" s="42" t="s">
         <v>51</v>
@@ -2069,24 +2132,27 @@
       <c r="K16" s="77"/>
       <c r="L16" s="77"/>
       <c r="M16" s="78"/>
-      <c r="N16" s="87"/>
+      <c r="N16" s="131"/>
       <c r="O16" s="79"/>
       <c r="P16" s="85"/>
       <c r="Q16" s="80"/>
-      <c r="R16" s="88"/>
+      <c r="R16" s="87"/>
       <c r="S16" s="81"/>
       <c r="T16" s="86"/>
-      <c r="U16" s="88"/>
-      <c r="V16" s="88"/>
-      <c r="W16" s="128">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="X16" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Y16" s="16"/>
+      <c r="U16" s="87"/>
+      <c r="V16" s="87"/>
+      <c r="W16" s="127">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="X16" s="82">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Y16" s="26" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
       <c r="AC16" s="42" t="s">
         <v>52</v>
       </c>
@@ -2105,24 +2171,28 @@
       <c r="K17" s="77"/>
       <c r="L17" s="77"/>
       <c r="M17" s="78"/>
-      <c r="N17" s="87"/>
+      <c r="N17" s="131"/>
       <c r="O17" s="79"/>
       <c r="P17" s="85"/>
       <c r="Q17" s="80"/>
-      <c r="R17" s="88"/>
+      <c r="R17" s="87"/>
       <c r="S17" s="81"/>
       <c r="T17" s="86"/>
-      <c r="U17" s="88"/>
-      <c r="V17" s="88"/>
-      <c r="W17" s="128">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="X17" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="AA17" s="89"/>
+      <c r="U17" s="87"/>
+      <c r="V17" s="87"/>
+      <c r="W17" s="127">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="X17" s="82">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Y17" s="26" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AA17" s="88"/>
       <c r="AC17" s="42" t="s">
         <v>53</v>
       </c>
@@ -2140,23 +2210,27 @@
       <c r="J18" s="84"/>
       <c r="K18" s="77"/>
       <c r="L18" s="77"/>
-      <c r="M18" s="91"/>
-      <c r="N18" s="87"/>
+      <c r="M18" s="90"/>
+      <c r="N18" s="131"/>
       <c r="O18" s="79"/>
       <c r="P18" s="85"/>
       <c r="Q18" s="80"/>
-      <c r="R18" s="88"/>
+      <c r="R18" s="87"/>
       <c r="S18" s="81"/>
       <c r="T18" s="86"/>
-      <c r="U18" s="88"/>
-      <c r="V18" s="88"/>
-      <c r="W18" s="128">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="X18" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
+      <c r="U18" s="87"/>
+      <c r="V18" s="87"/>
+      <c r="W18" s="127">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="X18" s="82">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Y18" s="26" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
       </c>
       <c r="AA18" s="82"/>
       <c r="AC18" s="26" t="s">
@@ -2177,69 +2251,70 @@
       <c r="K19" s="77"/>
       <c r="L19" s="77"/>
       <c r="M19" s="78"/>
-      <c r="N19" s="87"/>
+      <c r="N19" s="131"/>
       <c r="O19" s="79"/>
       <c r="P19" s="85"/>
       <c r="Q19" s="80"/>
-      <c r="R19" s="88"/>
+      <c r="R19" s="87"/>
       <c r="S19" s="81"/>
       <c r="T19" s="86"/>
-      <c r="U19" s="88"/>
-      <c r="V19" s="88"/>
-      <c r="W19" s="128">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="X19" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Z19" s="90"/>
+      <c r="U19" s="87"/>
+      <c r="V19" s="87"/>
+      <c r="W19" s="127">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="X19" s="82">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Y19" s="26" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="Z19" s="89"/>
       <c r="AC19" s="16" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:29">
-      <c r="A20" s="92"/>
-      <c r="B20" s="93" t="s">
+      <c r="A20" s="91"/>
+      <c r="B20" s="92" t="s">
         <v>56</v>
       </c>
-      <c r="C20" s="94"/>
-      <c r="D20" s="95"/>
+      <c r="C20" s="93"/>
+      <c r="D20" s="94"/>
       <c r="E20" s="72">
         <f>E19-C20+D20</f>
         <v>0</v>
       </c>
-      <c r="F20" s="96"/>
-      <c r="G20" s="97"/>
+      <c r="F20" s="95"/>
+      <c r="G20" s="96"/>
       <c r="H20" s="1"/>
-      <c r="I20" s="98"/>
-      <c r="J20" s="98"/>
-      <c r="K20" s="99"/>
-      <c r="L20" s="98"/>
-      <c r="M20" s="100"/>
+      <c r="I20" s="97"/>
+      <c r="J20" s="97"/>
+      <c r="K20" s="98"/>
+      <c r="L20" s="97"/>
+      <c r="M20" s="99"/>
       <c r="N20" s="1"/>
-      <c r="O20" s="101" t="s">
+      <c r="O20" s="100" t="s">
         <v>57</v>
       </c>
-      <c r="P20" s="99"/>
-      <c r="Q20" s="102"/>
-      <c r="R20" s="88">
+      <c r="P20" s="98"/>
+      <c r="Q20" s="101"/>
+      <c r="R20" s="87">
         <f>R19-P20+Q20-C20+D20</f>
         <v>0</v>
       </c>
-      <c r="S20" s="103"/>
-      <c r="T20" s="104"/>
-      <c r="U20" s="104"/>
+      <c r="S20" s="102"/>
+      <c r="T20" s="103"/>
+      <c r="U20" s="103"/>
       <c r="V20" s="40"/>
       <c r="W20" s="40"/>
-      <c r="X20" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="X20" s="82"/>
     </row>
     <row r="21" spans="1:29">
-      <c r="A21" s="92"/>
+      <c r="A21" s="91"/>
       <c r="B21" s="28"/>
       <c r="C21" s="29"/>
       <c r="D21" s="30"/>
@@ -2249,43 +2324,40 @@
       <c r="H21" s="31"/>
       <c r="I21" s="49"/>
       <c r="J21" s="49"/>
-      <c r="K21" s="105"/>
+      <c r="K21" s="104"/>
       <c r="L21" s="49"/>
       <c r="M21" s="50"/>
       <c r="N21" s="31"/>
       <c r="O21" s="34"/>
       <c r="P21" s="29"/>
       <c r="Q21" s="29"/>
-      <c r="R21" s="104"/>
-      <c r="S21" s="104"/>
-      <c r="T21" s="104"/>
-      <c r="U21" s="104"/>
+      <c r="R21" s="103"/>
+      <c r="S21" s="103"/>
+      <c r="T21" s="103"/>
+      <c r="U21" s="103"/>
       <c r="V21" s="29"/>
       <c r="W21" s="29"/>
-      <c r="X21" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="X21" s="82"/>
     </row>
     <row r="22" spans="1:29">
-      <c r="A22" s="92"/>
-      <c r="B22" s="106" t="s">
+      <c r="A22" s="91"/>
+      <c r="B22" s="105" t="s">
         <v>58</v>
       </c>
-      <c r="C22" s="107"/>
-      <c r="D22" s="108"/>
-      <c r="E22" s="107"/>
-      <c r="F22" s="109"/>
+      <c r="C22" s="106"/>
+      <c r="D22" s="107"/>
+      <c r="E22" s="106"/>
+      <c r="F22" s="108"/>
       <c r="G22" s="1"/>
       <c r="H22" s="1"/>
-      <c r="I22" s="98"/>
-      <c r="J22" s="98"/>
-      <c r="K22" s="99"/>
-      <c r="L22" s="98"/>
-      <c r="M22" s="100"/>
+      <c r="I22" s="97"/>
+      <c r="J22" s="97"/>
+      <c r="K22" s="98"/>
+      <c r="L22" s="97"/>
+      <c r="M22" s="99"/>
       <c r="N22" s="1"/>
-      <c r="O22" s="110"/>
-      <c r="P22" s="111">
+      <c r="O22" s="109"/>
+      <c r="P22" s="110">
         <f>R20-E20</f>
         <v>0</v>
       </c>
@@ -2296,13 +2368,10 @@
       <c r="U22" s="29"/>
       <c r="V22" s="29"/>
       <c r="W22" s="30"/>
-      <c r="X22" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="X22" s="82"/>
     </row>
     <row r="23" spans="1:29">
-      <c r="A23" s="92"/>
+      <c r="A23" s="91"/>
       <c r="B23" s="28"/>
       <c r="C23" s="29"/>
       <c r="D23" s="30"/>
@@ -2311,7 +2380,7 @@
       <c r="H23" s="31"/>
       <c r="I23" s="49"/>
       <c r="J23" s="49"/>
-      <c r="K23" s="105"/>
+      <c r="K23" s="104"/>
       <c r="L23" s="49"/>
       <c r="M23" s="50"/>
       <c r="N23" s="31"/>
@@ -2324,13 +2393,10 @@
       <c r="U23" s="29"/>
       <c r="V23" s="29"/>
       <c r="W23" s="30"/>
-      <c r="X23" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="X23" s="82"/>
     </row>
     <row r="24" spans="1:29">
-      <c r="A24" s="92"/>
+      <c r="A24" s="91"/>
       <c r="B24" s="28"/>
       <c r="C24" s="29"/>
       <c r="D24" s="30"/>
@@ -2339,7 +2405,7 @@
       <c r="H24" s="31"/>
       <c r="I24" s="49"/>
       <c r="J24" s="49"/>
-      <c r="K24" s="105"/>
+      <c r="K24" s="104"/>
       <c r="L24" s="49"/>
       <c r="M24" s="50"/>
       <c r="N24" s="31"/>
@@ -2357,14 +2423,11 @@
       <c r="U24" s="29"/>
       <c r="V24" s="29"/>
       <c r="W24" s="30"/>
-      <c r="X24" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="X24" s="82"/>
       <c r="Y24" s="16"/>
     </row>
     <row r="25" spans="1:29">
-      <c r="A25" s="92"/>
+      <c r="A25" s="91"/>
       <c r="B25" s="28"/>
       <c r="C25" s="29"/>
       <c r="D25" s="30"/>
@@ -2373,7 +2436,7 @@
       <c r="H25" s="31"/>
       <c r="I25" s="49"/>
       <c r="J25" s="49"/>
-      <c r="K25" s="105"/>
+      <c r="K25" s="104"/>
       <c r="L25" s="49"/>
       <c r="M25" s="50"/>
       <c r="N25" s="31"/>
@@ -2392,14 +2455,11 @@
       <c r="U25" s="29"/>
       <c r="V25" s="29"/>
       <c r="W25" s="30"/>
-      <c r="X25" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="X25" s="82"/>
       <c r="Y25" s="16"/>
     </row>
     <row r="26" spans="1:29">
-      <c r="A26" s="92"/>
+      <c r="A26" s="91"/>
       <c r="B26" s="28"/>
       <c r="C26" s="29"/>
       <c r="D26" s="30"/>
@@ -2408,15 +2468,15 @@
       <c r="H26" s="31"/>
       <c r="I26" s="49"/>
       <c r="J26" s="49"/>
-      <c r="K26" s="105"/>
+      <c r="K26" s="104"/>
       <c r="L26" s="49"/>
       <c r="M26" s="50"/>
       <c r="N26" s="31"/>
-      <c r="O26" s="112" t="str">
+      <c r="O26" s="111" t="str">
         <f>"Excesso de "&amp;AB3&amp;":"</f>
         <v>Excesso de execução:</v>
       </c>
-      <c r="P26" s="113">
+      <c r="P26" s="112">
         <f>ABS(P24-P25)</f>
         <v>0</v>
       </c>
@@ -2427,14 +2487,11 @@
       <c r="U26" s="29"/>
       <c r="V26" s="29"/>
       <c r="W26" s="30"/>
-      <c r="X26" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="X26" s="82"/>
       <c r="Y26" s="16"/>
     </row>
     <row r="27" spans="1:29">
-      <c r="A27" s="92"/>
+      <c r="A27" s="91"/>
       <c r="B27" s="28"/>
       <c r="C27" s="29"/>
       <c r="D27" s="30"/>
@@ -2443,7 +2500,7 @@
       <c r="H27" s="31"/>
       <c r="I27" s="49"/>
       <c r="J27" s="49"/>
-      <c r="K27" s="105"/>
+      <c r="K27" s="104"/>
       <c r="L27" s="49"/>
       <c r="M27" s="50"/>
       <c r="N27" s="31"/>
@@ -2458,345 +2515,246 @@
       <c r="U27" s="29"/>
       <c r="V27" s="29"/>
       <c r="W27" s="30"/>
-      <c r="X27" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="X27" s="82"/>
       <c r="Y27" s="16"/>
     </row>
     <row r="28" spans="1:29">
-      <c r="X28" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="X28" s="82"/>
       <c r="Y28" s="16"/>
     </row>
     <row r="29" spans="1:29">
-      <c r="B29" s="114" t="s">
+      <c r="B29" s="113" t="s">
         <v>61</v>
       </c>
-      <c r="C29" s="115"/>
-      <c r="D29" s="115"/>
-      <c r="E29" s="116">
+      <c r="C29" s="114"/>
+      <c r="D29" s="114"/>
+      <c r="E29" s="115">
         <f>E20</f>
         <v>0</v>
       </c>
-      <c r="O29" s="117" t="s">
+      <c r="O29" s="116" t="s">
         <v>62</v>
       </c>
-      <c r="P29" s="117"/>
-      <c r="Q29" s="117"/>
-      <c r="R29" s="115">
+      <c r="P29" s="116"/>
+      <c r="Q29" s="116"/>
+      <c r="R29" s="114">
         <f>R20</f>
         <v>0</v>
       </c>
-      <c r="X29" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="X29" s="82"/>
       <c r="Y29" s="16"/>
     </row>
     <row r="30" spans="1:29">
-      <c r="B30" s="114" t="s">
+      <c r="B30" s="113" t="s">
         <v>63</v>
       </c>
-      <c r="C30" s="115"/>
-      <c r="D30" s="115"/>
-      <c r="E30" s="118"/>
-      <c r="O30" s="114" t="s">
+      <c r="C30" s="114"/>
+      <c r="D30" s="114"/>
+      <c r="E30" s="117"/>
+      <c r="O30" s="113" t="s">
         <v>63</v>
       </c>
-      <c r="P30" s="117"/>
-      <c r="Q30" s="117"/>
-      <c r="R30" s="117">
+      <c r="P30" s="116"/>
+      <c r="Q30" s="116"/>
+      <c r="R30" s="116">
         <f>G30</f>
         <v>0</v>
       </c>
-      <c r="X30" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="X30" s="82"/>
       <c r="Y30" s="16"/>
     </row>
     <row r="31" spans="1:29">
-      <c r="B31" s="114" t="s">
+      <c r="B31" s="113" t="s">
         <v>65</v>
       </c>
-      <c r="C31" s="115"/>
-      <c r="D31" s="115"/>
-      <c r="E31" s="116">
+      <c r="C31" s="114"/>
+      <c r="D31" s="114"/>
+      <c r="E31" s="115">
         <f>E32-E29</f>
         <v>0</v>
       </c>
-      <c r="O31" s="114" t="s">
+      <c r="O31" s="113" t="s">
         <v>65</v>
       </c>
-      <c r="P31" s="117"/>
-      <c r="Q31" s="117"/>
-      <c r="R31" s="115">
+      <c r="P31" s="116"/>
+      <c r="Q31" s="116"/>
+      <c r="R31" s="114">
         <f>R32-R29</f>
         <v>0</v>
       </c>
-      <c r="X31" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="X31" s="82"/>
       <c r="Y31" s="16"/>
     </row>
     <row r="32" spans="1:29">
-      <c r="B32" s="114" t="s">
+      <c r="B32" s="113" t="s">
         <v>66</v>
       </c>
-      <c r="C32" s="115"/>
-      <c r="D32" s="115"/>
-      <c r="E32" s="116">
+      <c r="C32" s="114"/>
+      <c r="D32" s="114"/>
+      <c r="E32" s="115">
         <f>E29*E30</f>
         <v>0</v>
       </c>
-      <c r="O32" s="114" t="s">
+      <c r="O32" s="113" t="s">
         <v>67</v>
       </c>
-      <c r="P32" s="117"/>
-      <c r="Q32" s="117"/>
-      <c r="R32" s="115">
+      <c r="P32" s="116"/>
+      <c r="Q32" s="116"/>
+      <c r="R32" s="114">
         <f>R29*R30</f>
         <v>0</v>
       </c>
-      <c r="X32" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="X32" s="82"/>
       <c r="Y32" s="16"/>
     </row>
     <row r="33" spans="15:25">
-      <c r="O33" s="120"/>
-      <c r="P33" s="120"/>
-      <c r="Q33" s="120"/>
-      <c r="R33" s="121"/>
-      <c r="X33" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="O33" s="119"/>
+      <c r="P33" s="119"/>
+      <c r="Q33" s="119"/>
+      <c r="R33" s="120"/>
+      <c r="X33" s="82"/>
       <c r="Y33" s="16"/>
     </row>
     <row r="34" spans="15:25">
-      <c r="O34" s="123" t="s">
+      <c r="O34" s="122" t="s">
         <v>71</v>
       </c>
-      <c r="P34" s="123"/>
-      <c r="Q34" s="123"/>
-      <c r="R34" s="124">
+      <c r="P34" s="122"/>
+      <c r="Q34" s="122"/>
+      <c r="R34" s="123">
         <f>ABS(E32-R32)</f>
         <v>0</v>
       </c>
-      <c r="X34" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="X34" s="82"/>
       <c r="Y34" s="16"/>
     </row>
     <row r="35" spans="15:25">
-      <c r="O35" s="125" t="s">
+      <c r="O35" s="124" t="s">
         <v>60</v>
       </c>
-      <c r="P35" s="117"/>
-      <c r="Q35" s="117"/>
-      <c r="R35" s="115"/>
-      <c r="X35" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="P35" s="116"/>
+      <c r="Q35" s="116"/>
+      <c r="R35" s="114"/>
+      <c r="X35" s="82"/>
       <c r="Y35" s="16"/>
     </row>
     <row r="36" spans="15:25">
-      <c r="X36" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="X36" s="82"/>
       <c r="Y36" s="16"/>
     </row>
     <row r="37" spans="15:25">
-      <c r="O37" s="126" t="str">
+      <c r="O37" s="125" t="str">
         <f>"Excesso utilizado na operação nº xxxx - Anexo "</f>
         <v xml:space="preserve">Excesso utilizado na operação nº xxxx - Anexo </v>
       </c>
-      <c r="X37" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="X37" s="82"/>
       <c r="Y37" s="16"/>
     </row>
     <row r="38" spans="15:25">
-      <c r="X38" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="X38" s="82"/>
       <c r="Y38" s="16"/>
     </row>
     <row r="39" spans="15:25">
-      <c r="X39" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="X39" s="82"/>
       <c r="Y39" s="16"/>
     </row>
     <row r="40" spans="15:25">
-      <c r="X40" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="X40" s="82"/>
       <c r="Y40" s="16"/>
     </row>
     <row r="41" spans="15:25">
-      <c r="X41" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="X41" s="82"/>
       <c r="Y41" s="16"/>
     </row>
     <row r="42" spans="15:25">
-      <c r="X42" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="X42" s="82"/>
       <c r="Y42" s="16"/>
     </row>
     <row r="43" spans="15:25">
-      <c r="X43" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="X43" s="82"/>
       <c r="Y43" s="16"/>
     </row>
     <row r="44" spans="15:25">
-      <c r="X44" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="X44" s="82"/>
       <c r="Y44" s="16"/>
     </row>
     <row r="45" spans="15:25">
-      <c r="X45" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="X45" s="82"/>
       <c r="Y45" s="16"/>
     </row>
     <row r="46" spans="15:25">
-      <c r="X46" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="X46" s="82"/>
       <c r="Y46" s="16"/>
     </row>
     <row r="47" spans="15:25">
-      <c r="X47" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="X47" s="82"/>
       <c r="Y47" s="16"/>
     </row>
     <row r="48" spans="15:25">
-      <c r="X48" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="X48" s="82"/>
       <c r="Y48" s="16"/>
     </row>
     <row r="49" spans="24:25">
-      <c r="X49" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="X49" s="82"/>
       <c r="Y49" s="16"/>
     </row>
     <row r="50" spans="24:25">
-      <c r="X50" s="82" t="e">
-        <f>#REF!-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="X50" s="82"/>
       <c r="Y50" s="16"/>
     </row>
     <row r="51" spans="24:25">
-      <c r="X51" s="82">
-        <f t="shared" ref="X51:X57" si="1">V13-Q13</f>
-        <v>0</v>
-      </c>
+      <c r="X51" s="82"/>
       <c r="Y51" s="16"/>
     </row>
     <row r="52" spans="24:25">
-      <c r="X52" s="82">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="X52" s="82"/>
       <c r="Y52" s="16"/>
     </row>
     <row r="53" spans="24:25">
-      <c r="X53" s="82">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="X53" s="82"/>
       <c r="Y53" s="16"/>
     </row>
     <row r="54" spans="24:25">
-      <c r="X54" s="82">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="X54" s="82"/>
       <c r="Y54" s="16"/>
     </row>
     <row r="55" spans="24:25">
-      <c r="X55" s="82">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="X55" s="82"/>
       <c r="Y55" s="16"/>
     </row>
     <row r="56" spans="24:25">
-      <c r="X56" s="82">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="X56" s="82"/>
       <c r="Y56" s="16"/>
     </row>
     <row r="57" spans="24:25">
-      <c r="X57" s="82">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="X57" s="82"/>
       <c r="Y57" s="16"/>
-    </row>
-    <row r="58" spans="24:25">
-      <c r="X58" s="25" t="e">
-        <f>SUM(X13:X57)</f>
-        <v>#REF!</v>
-      </c>
     </row>
     <row r="60" spans="24:25" ht="13.5" hidden="1" customHeight="1"/>
     <row r="61" spans="24:25" ht="13.5" hidden="1" customHeight="1"/>
     <row r="68" spans="25:26">
-      <c r="Y68" s="119" t="s">
+      <c r="Y68" s="118" t="s">
         <v>64</v>
       </c>
-      <c r="Z68" s="119"/>
+      <c r="Z68" s="118"/>
     </row>
     <row r="69" spans="25:26">
-      <c r="Y69" s="119"/>
-      <c r="Z69" s="119"/>
+      <c r="Y69" s="118"/>
+      <c r="Z69" s="118"/>
     </row>
     <row r="70" spans="25:26">
-      <c r="Y70" s="119" t="s">
+      <c r="Y70" s="118" t="s">
         <v>68</v>
       </c>
-      <c r="Z70" s="119" t="s">
+      <c r="Z70" s="118" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="71" spans="25:26">
-      <c r="Y71" s="119" t="s">
+      <c r="Y71" s="118" t="s">
         <v>70</v>
       </c>
-      <c r="Z71" s="122" t="str">
+      <c r="Z71" s="121" t="str">
         <f>A1</f>
         <v>Recálculo da operação nº 409.906.274 - Capitalização Afastada</v>
       </c>

</xml_diff>